<commit_message>
sync: stock y precios actualizados mié 09/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -8985,7 +8985,7 @@
         <v>871</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>376</v>
+        <v>140</v>
       </c>
       <c r="D406" s="0">
         <v>857.67</v>
@@ -9268,7 +9268,7 @@
         <v>45</v>
       </c>
       <c r="D426" s="0">
-        <v>4399.56</v>
+        <v>4708</v>
       </c>
     </row>
     <row r="427">

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb 12/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="1087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="1089">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -2859,6 +2859,12 @@
   </si>
   <si>
     <t>SUPER-O 100 MG X 100 COMP - 000024653</t>
+  </si>
+  <si>
+    <t>000024713</t>
+  </si>
+  <si>
+    <t>SUPER-O 100mg Comp. Rec. x 20 - 000024713</t>
   </si>
   <si>
     <t>000009961</t>
@@ -3338,7 +3344,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D508"/>
+  <dimension ref="A2:D509"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -9517,10 +9523,10 @@
         <v>950</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D444" s="0">
-        <v>266200</v>
+        <v>3340</v>
       </c>
     </row>
     <row r="445">
@@ -9534,7 +9540,7 @@
         <v>92</v>
       </c>
       <c r="D445" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="446">
@@ -9548,7 +9554,7 @@
         <v>92</v>
       </c>
       <c r="D446" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="447">
@@ -9559,24 +9565,24 @@
         <v>956</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>957</v>
+        <v>92</v>
       </c>
       <c r="D447" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="0" t="s">
+        <v>957</v>
+      </c>
+      <c r="B448" s="0" t="s">
         <v>958</v>
       </c>
-      <c r="B448" s="0" t="s">
+      <c r="C448" s="0" t="s">
         <v>959</v>
       </c>
-      <c r="C448" s="0" t="s">
-        <v>957</v>
-      </c>
       <c r="D448" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="449">
@@ -9587,10 +9593,10 @@
         <v>961</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>957</v>
+        <v>959</v>
       </c>
       <c r="D449" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="450">
@@ -9601,10 +9607,10 @@
         <v>963</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>957</v>
+        <v>959</v>
       </c>
       <c r="D450" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="451">
@@ -9615,10 +9621,10 @@
         <v>965</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>957</v>
+        <v>959</v>
       </c>
       <c r="D451" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="452">
@@ -9629,10 +9635,10 @@
         <v>967</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>70</v>
+        <v>959</v>
       </c>
       <c r="D452" s="0">
-        <v>4276</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="453">
@@ -9643,10 +9649,10 @@
         <v>969</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="D453" s="0">
-        <v>3930</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="454">
@@ -9657,10 +9663,10 @@
         <v>971</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D454" s="0">
-        <v>4392.3</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="455">
@@ -9671,24 +9677,24 @@
         <v>973</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>974</v>
+        <v>92</v>
       </c>
       <c r="D455" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="0" t="s">
+        <v>974</v>
+      </c>
+      <c r="B456" s="0" t="s">
         <v>975</v>
       </c>
-      <c r="B456" s="0" t="s">
+      <c r="C456" s="0" t="s">
         <v>976</v>
       </c>
-      <c r="C456" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D456" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="457">
@@ -9702,7 +9708,7 @@
         <v>52</v>
       </c>
       <c r="D457" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="458">
@@ -9716,7 +9722,7 @@
         <v>52</v>
       </c>
       <c r="D458" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="459">
@@ -9727,10 +9733,10 @@
         <v>982</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>376</v>
+        <v>52</v>
       </c>
       <c r="D459" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="460">
@@ -9744,7 +9750,7 @@
         <v>376</v>
       </c>
       <c r="D460" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="461">
@@ -9755,10 +9761,10 @@
         <v>986</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="D461" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="462">
@@ -9769,10 +9775,10 @@
         <v>988</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D462" s="0">
-        <v>12000</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="463">
@@ -9786,7 +9792,7 @@
         <v>52</v>
       </c>
       <c r="D463" s="0">
-        <v>17425</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="464">
@@ -9797,66 +9803,66 @@
         <v>992</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>993</v>
+        <v>52</v>
       </c>
       <c r="D464" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
+        <v>993</v>
+      </c>
+      <c r="B465" s="0" t="s">
         <v>994</v>
       </c>
-      <c r="B465" s="0" t="s">
+      <c r="C465" s="0" t="s">
         <v>995</v>
       </c>
-      <c r="C465" s="0" t="s">
-        <v>996</v>
-      </c>
       <c r="D465" s="0">
-        <v>2282.3</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
+        <v>996</v>
+      </c>
+      <c r="B466" s="0" t="s">
         <v>997</v>
       </c>
-      <c r="B466" s="0" t="s">
+      <c r="C466" s="0" t="s">
         <v>998</v>
       </c>
-      <c r="C466" s="0" t="s">
-        <v>999</v>
-      </c>
       <c r="D466" s="0">
-        <v>386</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="0" t="s">
+        <v>999</v>
+      </c>
+      <c r="B467" s="0" t="s">
         <v>1000</v>
       </c>
-      <c r="B467" s="0" t="s">
+      <c r="C467" s="0" t="s">
         <v>1001</v>
       </c>
-      <c r="C467" s="0" t="s">
-        <v>1002</v>
-      </c>
       <c r="D467" s="0">
-        <v>385.4</v>
+        <v>386</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="0" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B468" s="0" t="s">
         <v>1003</v>
       </c>
-      <c r="B468" s="0" t="s">
+      <c r="C468" s="0" t="s">
         <v>1004</v>
       </c>
-      <c r="C468" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D468" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="469">
@@ -9867,10 +9873,10 @@
         <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>123</v>
+        <v>92</v>
       </c>
       <c r="D469" s="0">
-        <v>1890</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="470">
@@ -9881,10 +9887,10 @@
         <v>1008</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>580</v>
+        <v>123</v>
       </c>
       <c r="D470" s="0">
-        <v>71176.4</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="471">
@@ -9895,10 +9901,10 @@
         <v>1010</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>140</v>
+        <v>580</v>
       </c>
       <c r="D471" s="0">
-        <v>87</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="472">
@@ -9909,10 +9915,10 @@
         <v>1012</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="D472" s="0">
-        <v>950</v>
+        <v>87</v>
       </c>
     </row>
     <row r="473">
@@ -9923,10 +9929,10 @@
         <v>1014</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>469</v>
+        <v>70</v>
       </c>
       <c r="D473" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="474">
@@ -9937,10 +9943,10 @@
         <v>1016</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>160</v>
+        <v>469</v>
       </c>
       <c r="D474" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="475">
@@ -9951,10 +9957,10 @@
         <v>1018</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>478</v>
+        <v>160</v>
       </c>
       <c r="D475" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="476">
@@ -9965,10 +9971,10 @@
         <v>1020</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>70</v>
+        <v>478</v>
       </c>
       <c r="D476" s="0">
-        <v>5790</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="477">
@@ -9979,10 +9985,10 @@
         <v>1022</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>919</v>
+        <v>70</v>
       </c>
       <c r="D477" s="0">
-        <v>880</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="478">
@@ -10021,10 +10027,10 @@
         <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>21</v>
+        <v>919</v>
       </c>
       <c r="D480" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="481">
@@ -10035,10 +10041,10 @@
         <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D481" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="482">
@@ -10052,7 +10058,7 @@
         <v>15</v>
       </c>
       <c r="D482" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="483">
@@ -10063,10 +10069,10 @@
         <v>1034</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D483" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="484">
@@ -10080,7 +10086,7 @@
         <v>281</v>
       </c>
       <c r="D484" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="485">
@@ -10091,10 +10097,10 @@
         <v>1038</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D485" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="486">
@@ -10108,7 +10114,7 @@
         <v>15</v>
       </c>
       <c r="D486" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="487">
@@ -10119,24 +10125,24 @@
         <v>1042</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>1043</v>
+        <v>15</v>
       </c>
       <c r="D487" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="0" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B488" s="0" t="s">
         <v>1044</v>
       </c>
-      <c r="B488" s="0" t="s">
+      <c r="C488" s="0" t="s">
         <v>1045</v>
       </c>
-      <c r="C488" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D488" s="0">
-        <v>14819</v>
+        <v>1</v>
       </c>
     </row>
     <row r="489">
@@ -10147,10 +10153,10 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>376</v>
+        <v>28</v>
       </c>
       <c r="D489" s="0">
-        <v>3859.93</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="490">
@@ -10164,7 +10170,7 @@
         <v>376</v>
       </c>
       <c r="D490" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="491">
@@ -10175,10 +10181,10 @@
         <v>1051</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D491" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="492">
@@ -10192,7 +10198,7 @@
         <v>338</v>
       </c>
       <c r="D492" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="493">
@@ -10203,10 +10209,10 @@
         <v>1055</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>37</v>
+        <v>338</v>
       </c>
       <c r="D493" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="494">
@@ -10217,24 +10223,24 @@
         <v>1057</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>1058</v>
+        <v>37</v>
       </c>
       <c r="D494" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="0" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B495" s="0" t="s">
         <v>1059</v>
       </c>
-      <c r="B495" s="0" t="s">
+      <c r="C495" s="0" t="s">
         <v>1060</v>
       </c>
-      <c r="C495" s="0" t="s">
-        <v>105</v>
-      </c>
       <c r="D495" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="496">
@@ -10245,10 +10251,10 @@
         <v>1062</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D496" s="0">
-        <v>43590.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="497">
@@ -10259,10 +10265,10 @@
         <v>1064</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>469</v>
+        <v>92</v>
       </c>
       <c r="D497" s="0">
-        <v>207558.07</v>
+        <v>43590.25</v>
       </c>
     </row>
     <row r="498">
@@ -10273,10 +10279,10 @@
         <v>1066</v>
       </c>
       <c r="C498" s="0" t="s">
-        <v>376</v>
+        <v>469</v>
       </c>
       <c r="D498" s="0">
-        <v>77429.29</v>
+        <v>207558.07</v>
       </c>
     </row>
     <row r="499">
@@ -10290,7 +10296,7 @@
         <v>376</v>
       </c>
       <c r="D499" s="0">
-        <v>42913.42</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="500">
@@ -10304,7 +10310,7 @@
         <v>376</v>
       </c>
       <c r="D500" s="0">
-        <v>88806.25</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="501">
@@ -10318,7 +10324,7 @@
         <v>376</v>
       </c>
       <c r="D501" s="0">
-        <v>50781.52</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="502">
@@ -10329,10 +10335,10 @@
         <v>1074</v>
       </c>
       <c r="C502" s="0" t="s">
-        <v>21</v>
+        <v>376</v>
       </c>
       <c r="D502" s="0">
-        <v>1600</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="503">
@@ -10343,10 +10349,10 @@
         <v>1076</v>
       </c>
       <c r="C503" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D503" s="0">
-        <v>3455.8</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="504">
@@ -10360,7 +10366,7 @@
         <v>28</v>
       </c>
       <c r="D504" s="0">
-        <v>3987</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="505">
@@ -10374,7 +10380,7 @@
         <v>28</v>
       </c>
       <c r="D505" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="506">
@@ -10388,7 +10394,7 @@
         <v>28</v>
       </c>
       <c r="D506" s="0">
-        <v>3382.65</v>
+        <v>4010.17</v>
       </c>
     </row>
     <row r="507">
@@ -10399,10 +10405,10 @@
         <v>1084</v>
       </c>
       <c r="C507" s="0" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="D507" s="0">
-        <v>430</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="508">
@@ -10413,9 +10419,23 @@
         <v>1086</v>
       </c>
       <c r="C508" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D508" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="0" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B509" s="0" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C509" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="D508" s="0">
+      <c r="D509" s="0">
         <v>465</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados jue 17/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3492,7 +3492,7 @@
         <v>28</v>
       </c>
       <c r="D13" s="0">
-        <v>134.59</v>
+        <v>139.48</v>
       </c>
     </row>
     <row r="14">
@@ -3674,7 +3674,7 @@
         <v>28</v>
       </c>
       <c r="D26" s="0">
-        <v>160.14</v>
+        <v>162.86</v>
       </c>
     </row>
     <row r="27">
@@ -4304,7 +4304,7 @@
         <v>52</v>
       </c>
       <c r="D71" s="0">
-        <v>1075</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="72">
@@ -4472,7 +4472,7 @@
         <v>52</v>
       </c>
       <c r="D83" s="0">
-        <v>330</v>
+        <v>362</v>
       </c>
     </row>
     <row r="84">
@@ -5102,7 +5102,7 @@
         <v>28</v>
       </c>
       <c r="D128" s="0">
-        <v>7118.9</v>
+        <v>7377.5</v>
       </c>
     </row>
     <row r="129">
@@ -5312,7 +5312,7 @@
         <v>52</v>
       </c>
       <c r="D143" s="0">
-        <v>1800</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="144">
@@ -5326,7 +5326,7 @@
         <v>52</v>
       </c>
       <c r="D144" s="0">
-        <v>2060</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="145">
@@ -5508,7 +5508,7 @@
         <v>28</v>
       </c>
       <c r="D157" s="0">
-        <v>103000</v>
+        <v>106950.8</v>
       </c>
     </row>
     <row r="158">
@@ -5522,7 +5522,7 @@
         <v>28</v>
       </c>
       <c r="D158" s="0">
-        <v>114000</v>
+        <v>118372.7</v>
       </c>
     </row>
     <row r="159">
@@ -5536,7 +5536,7 @@
         <v>28</v>
       </c>
       <c r="D159" s="0">
-        <v>135000</v>
+        <v>140178.2</v>
       </c>
     </row>
     <row r="160">
@@ -5718,7 +5718,7 @@
         <v>28</v>
       </c>
       <c r="D172" s="0">
-        <v>954.8</v>
+        <v>972.9</v>
       </c>
     </row>
     <row r="173">
@@ -5746,7 +5746,7 @@
         <v>28</v>
       </c>
       <c r="D174" s="0">
-        <v>2743.71</v>
+        <v>2908.78</v>
       </c>
     </row>
     <row r="175">
@@ -5760,7 +5760,7 @@
         <v>392</v>
       </c>
       <c r="D175" s="0">
-        <v>81</v>
+        <v>61</v>
       </c>
     </row>
     <row r="176">
@@ -5970,7 +5970,7 @@
         <v>28</v>
       </c>
       <c r="D190" s="0">
-        <v>9041.55</v>
+        <v>9748.5</v>
       </c>
     </row>
     <row r="191">
@@ -6558,7 +6558,7 @@
         <v>52</v>
       </c>
       <c r="D232" s="0">
-        <v>500</v>
+        <v>597</v>
       </c>
     </row>
     <row r="233">
@@ -6572,7 +6572,7 @@
         <v>52</v>
       </c>
       <c r="D233" s="0">
-        <v>210</v>
+        <v>223</v>
       </c>
     </row>
     <row r="234">
@@ -6712,7 +6712,7 @@
         <v>28</v>
       </c>
       <c r="D243" s="0">
-        <v>13636.84</v>
+        <v>14608.16</v>
       </c>
     </row>
     <row r="244">
@@ -7496,7 +7496,7 @@
         <v>28</v>
       </c>
       <c r="D299" s="0">
-        <v>7372.42</v>
+        <v>7655.2</v>
       </c>
     </row>
     <row r="300">
@@ -8392,7 +8392,7 @@
         <v>140</v>
       </c>
       <c r="D363" s="0">
-        <v>1229</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="364">
@@ -8406,7 +8406,7 @@
         <v>140</v>
       </c>
       <c r="D364" s="0">
-        <v>4500</v>
+        <v>4712</v>
       </c>
     </row>
     <row r="365">
@@ -8434,7 +8434,7 @@
         <v>28</v>
       </c>
       <c r="D366" s="0">
-        <v>1945.1</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="367">
@@ -8938,7 +8938,7 @@
         <v>52</v>
       </c>
       <c r="D402" s="0">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="403">
@@ -8952,7 +8952,7 @@
         <v>28</v>
       </c>
       <c r="D403" s="0">
-        <v>714.74</v>
+        <v>740.7</v>
       </c>
     </row>
     <row r="404">
@@ -9316,7 +9316,7 @@
         <v>919</v>
       </c>
       <c r="D429" s="0">
-        <v>580</v>
+        <v>626</v>
       </c>
     </row>
     <row r="430">
@@ -9330,7 +9330,7 @@
         <v>919</v>
       </c>
       <c r="D430" s="0">
-        <v>580</v>
+        <v>626</v>
       </c>
     </row>
     <row r="431">
@@ -9344,7 +9344,7 @@
         <v>919</v>
       </c>
       <c r="D431" s="0">
-        <v>580</v>
+        <v>626</v>
       </c>
     </row>
     <row r="432">
@@ -9708,7 +9708,7 @@
         <v>52</v>
       </c>
       <c r="D457" s="0">
-        <v>1200</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="458">
@@ -9722,7 +9722,7 @@
         <v>52</v>
       </c>
       <c r="D458" s="0">
-        <v>278</v>
+        <v>298</v>
       </c>
     </row>
     <row r="459">
@@ -9736,7 +9736,7 @@
         <v>52</v>
       </c>
       <c r="D459" s="0">
-        <v>562</v>
+        <v>596</v>
       </c>
     </row>
     <row r="460">
@@ -10156,7 +10156,7 @@
         <v>28</v>
       </c>
       <c r="D489" s="0">
-        <v>14819</v>
+        <v>15189</v>
       </c>
     </row>
     <row r="490">
@@ -10366,7 +10366,7 @@
         <v>28</v>
       </c>
       <c r="D504" s="0">
-        <v>3455.8</v>
+        <v>3521.4</v>
       </c>
     </row>
     <row r="505">
@@ -10394,7 +10394,7 @@
         <v>28</v>
       </c>
       <c r="D506" s="0">
-        <v>4010.17</v>
+        <v>4086.37</v>
       </c>
     </row>
     <row r="507">

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb 19/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="1089">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="1092">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -1806,6 +1806,15 @@
   </si>
   <si>
     <t>JERINGA 1 ML EUROMIX - 000024331</t>
+  </si>
+  <si>
+    <t>DJE00515</t>
+  </si>
+  <si>
+    <t>JERINGA 1 ML X 1 - SM - DJE00515</t>
+  </si>
+  <si>
+    <t>SM</t>
   </si>
   <si>
     <t>000024702</t>
@@ -3344,7 +3353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D509"/>
+  <dimension ref="A2:D510"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -7146,7 +7155,7 @@
         <v>600</v>
       </c>
       <c r="D274" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="275">
@@ -7157,7 +7166,7 @@
         <v>602</v>
       </c>
       <c r="C275" s="0" t="s">
-        <v>52</v>
+        <v>603</v>
       </c>
       <c r="D275" s="0">
         <v>65</v>
@@ -7165,97 +7174,97 @@
     </row>
     <row r="276">
       <c r="A276" s="0" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B276" s="0" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C276" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D276" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="0" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B277" s="0" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C277" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D277" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="0" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B278" s="0" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C278" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D278" s="0">
-        <v>54.8</v>
+        <v>33</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="0" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B279" s="0" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C279" s="0" t="s">
-        <v>338</v>
+        <v>52</v>
       </c>
       <c r="D279" s="0">
-        <v>300</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="0" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B280" s="0" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C280" s="0" t="s">
         <v>338</v>
       </c>
       <c r="D280" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="0" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B281" s="0" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C281" s="0" t="s">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="D281" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="0" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B282" s="0" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C282" s="0" t="s">
-        <v>37</v>
+        <v>359</v>
       </c>
       <c r="D282" s="0">
         <v>450</v>
@@ -7263,13 +7272,13 @@
     </row>
     <row r="283">
       <c r="A283" s="0" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B283" s="0" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C283" s="0" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D283" s="0">
         <v>450</v>
@@ -7277,296 +7286,296 @@
     </row>
     <row r="284">
       <c r="A284" s="0" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B284" s="0" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C284" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D284" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="0" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B285" s="0" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C285" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D285" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="0" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B286" s="0" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="C286" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D286" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="0" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B287" s="0" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C287" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D287" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="0" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B288" s="0" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C288" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D288" s="0">
-        <v>1500</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="0" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B289" s="0" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C289" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D289" s="0">
-        <v>2600</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="0" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B290" s="0" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C290" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D290" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="0" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B291" s="0" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="C291" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D291" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="0" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B292" s="0" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C292" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D292" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="0" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B293" s="0" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C293" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D293" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="0" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B294" s="0" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C294" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D294" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="0" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B295" s="0" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C295" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D295" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="0" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B296" s="0" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C296" s="0" t="s">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="D296" s="0">
-        <v>4590</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="0" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B297" s="0" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C297" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D297" s="0">
-        <v>2300</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="0" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B298" s="0" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C298" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D298" s="0">
-        <v>1150</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="0" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B299" s="0" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C299" s="0" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="D299" s="0">
-        <v>7655.2</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="0" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B300" s="0" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C300" s="0" t="s">
-        <v>123</v>
+        <v>28</v>
       </c>
       <c r="D300" s="0">
-        <v>1790</v>
+        <v>7655.2</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="0" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B301" s="0" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C301" s="0" t="s">
         <v>123</v>
       </c>
       <c r="D301" s="0">
-        <v>3016.53</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="0" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B302" s="0" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C302" s="0" t="s">
         <v>123</v>
       </c>
       <c r="D302" s="0">
-        <v>4800</v>
+        <v>3016.53</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="0" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B303" s="0" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C303" s="0" t="s">
         <v>123</v>
       </c>
       <c r="D303" s="0">
-        <v>4450</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="0" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B304" s="0" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="C304" s="0" t="s">
-        <v>661</v>
+        <v>123</v>
       </c>
       <c r="D304" s="0">
-        <v>0</v>
+        <v>4450</v>
       </c>
     </row>
     <row r="305">
@@ -7577,130 +7586,130 @@
         <v>663</v>
       </c>
       <c r="C305" s="0" t="s">
-        <v>28</v>
+        <v>664</v>
       </c>
       <c r="D305" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="0" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B306" s="0" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="C306" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D306" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="0" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B307" s="0" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="D307" s="0">
-        <v>33940.5</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="0" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B308" s="0" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C308" s="0" t="s">
         <v>92</v>
       </c>
       <c r="D308" s="0">
-        <v>4525.4</v>
+        <v>33940.5</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="0" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B309" s="0" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="D309" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="0" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B310" s="0" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="D310" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="0" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B311" s="0" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D311" s="0">
-        <v>332750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="0" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B312" s="0" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>202</v>
+        <v>92</v>
       </c>
       <c r="D312" s="0">
-        <v>17440</v>
+        <v>332750</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="0" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B313" s="0" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C313" s="0" t="s">
         <v>202</v>
       </c>
       <c r="D313" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="0" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B314" s="0" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C314" s="0" t="s">
         <v>202</v>
@@ -7711,128 +7720,128 @@
     </row>
     <row r="315">
       <c r="A315" s="0" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B315" s="0" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>281</v>
+        <v>202</v>
       </c>
       <c r="D315" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="0" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="B316" s="0" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>202</v>
+        <v>281</v>
       </c>
       <c r="D316" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="0" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B317" s="0" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D317" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="0" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B318" s="0" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>92</v>
+        <v>207</v>
       </c>
       <c r="D318" s="0">
-        <v>25289</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="0" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B319" s="0" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C319" s="0" t="s">
         <v>92</v>
       </c>
       <c r="D319" s="0">
-        <v>252890</v>
+        <v>25289</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="0" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B320" s="0" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="D320" s="0">
-        <v>160</v>
+        <v>252890</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="0" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B321" s="0" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C321" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D321" s="0">
-        <v>285.6</v>
+        <v>160</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="0" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B322" s="0" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C322" s="0" t="s">
         <v>21</v>
       </c>
       <c r="D322" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="0" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B323" s="0" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>700</v>
+        <v>21</v>
       </c>
       <c r="D323" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="324">
@@ -7857,245 +7866,245 @@
         <v>705</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>15</v>
+        <v>706</v>
       </c>
       <c r="D325" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="0" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B326" s="0" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D326" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="0" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B327" s="0" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D327" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="0" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B328" s="0" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>151</v>
+        <v>15</v>
       </c>
       <c r="D328" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="0" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B329" s="0" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>281</v>
+        <v>151</v>
       </c>
       <c r="D329" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="0" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B330" s="0" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C330" s="0" t="s">
         <v>281</v>
       </c>
       <c r="D330" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="0" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B331" s="0" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>140</v>
+        <v>281</v>
       </c>
       <c r="D331" s="0">
-        <v>890</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="0" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B332" s="0" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C332" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D332" s="0">
-        <v>594</v>
+        <v>890</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="0" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B333" s="0" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C333" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D333" s="0">
-        <v>65</v>
+        <v>594</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="0" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B334" s="0" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D334" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="0" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B335" s="0" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="D335" s="0">
-        <v>420</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="0" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B336" s="0" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>359</v>
+        <v>34</v>
       </c>
       <c r="D336" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="0" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B337" s="0" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>21</v>
+        <v>359</v>
       </c>
       <c r="D337" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="0" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="B338" s="0" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D338" s="0">
-        <v>5780.66</v>
+        <v>377</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="0" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B339" s="0" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D339" s="0">
-        <v>898</v>
+        <v>5780.66</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="0" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B340" s="0" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>123</v>
+        <v>70</v>
       </c>
       <c r="D340" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="0" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B341" s="0" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>34</v>
+        <v>123</v>
       </c>
       <c r="D341" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="0" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B342" s="0" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D342" s="0">
         <v>650</v>
@@ -8103,44 +8112,44 @@
     </row>
     <row r="343">
       <c r="A343" s="0" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B343" s="0" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D343" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="0" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B344" s="0" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D344" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="0" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B345" s="0" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>746</v>
+        <v>92</v>
       </c>
       <c r="D345" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="346">
@@ -8151,326 +8160,326 @@
         <v>748</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>151</v>
+        <v>749</v>
       </c>
       <c r="D346" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="0" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B347" s="0" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>21</v>
+        <v>151</v>
       </c>
       <c r="D347" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="0" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B348" s="0" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D348" s="0">
-        <v>59000</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="0" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B349" s="0" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>151</v>
+        <v>34</v>
       </c>
       <c r="D349" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="0" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B350" s="0" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="C350" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D350" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="0" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B351" s="0" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="C351" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D351" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="0" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="B352" s="0" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="C352" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D352" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="0" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="B353" s="0" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="C353" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D353" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="0" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="B354" s="0" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>261</v>
+        <v>151</v>
       </c>
       <c r="D354" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="0" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="B355" s="0" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>140</v>
+        <v>261</v>
       </c>
       <c r="D355" s="0">
-        <v>350</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="0" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B356" s="0" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>281</v>
+        <v>140</v>
       </c>
       <c r="D356" s="0">
-        <v>1450</v>
+        <v>350</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="0" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B357" s="0" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>92</v>
+        <v>281</v>
       </c>
       <c r="D357" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="0" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B358" s="0" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="D358" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="0" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="B359" s="0" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D359" s="0">
-        <v>566</v>
+        <v>900</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="0" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="B360" s="0" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>469</v>
+        <v>281</v>
       </c>
       <c r="D360" s="0">
-        <v>64925</v>
+        <v>566</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="0" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="B361" s="0" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>15</v>
+        <v>469</v>
       </c>
       <c r="D361" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="0" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B362" s="0" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D362" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="0" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="B363" s="0" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>140</v>
+        <v>21</v>
       </c>
       <c r="D363" s="0">
-        <v>1269</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="0" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="B364" s="0" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="C364" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D364" s="0">
-        <v>4712</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="0" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="B365" s="0" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C365" s="0" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="D365" s="0">
-        <v>1250</v>
+        <v>4712</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="0" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="B366" s="0" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="C366" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D366" s="0">
-        <v>1986</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="0" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="B367" s="0" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D367" s="0">
-        <v>450</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="0" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B368" s="0" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="C368" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D368" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="0" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="B369" s="0" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
         <v>15</v>
@@ -8481,83 +8490,83 @@
     </row>
     <row r="370">
       <c r="A370" s="0" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="B370" s="0" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>379</v>
+        <v>15</v>
       </c>
       <c r="D370" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="0" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="B371" s="0" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="C371" s="0" t="s">
         <v>379</v>
       </c>
       <c r="D371" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="0" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B372" s="0" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>70</v>
+        <v>379</v>
       </c>
       <c r="D372" s="0">
-        <v>3427</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="0" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="B373" s="0" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C373" s="0" t="s">
         <v>70</v>
       </c>
       <c r="D373" s="0">
-        <v>10618</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="0" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B374" s="0" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>281</v>
+        <v>70</v>
       </c>
       <c r="D374" s="0">
-        <v>515</v>
+        <v>10618</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="0" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="B375" s="0" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>37</v>
+        <v>281</v>
       </c>
       <c r="D375" s="0">
         <v>515</v>
@@ -8565,86 +8574,86 @@
     </row>
     <row r="376">
       <c r="A376" s="0" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="B376" s="0" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D376" s="0">
-        <v>10000</v>
+        <v>515</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="0" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="B377" s="0" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>469</v>
+        <v>52</v>
       </c>
       <c r="D377" s="0">
-        <v>207558.08</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="0" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="B378" s="0" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="C378" s="0" t="s">
         <v>469</v>
       </c>
       <c r="D378" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="0" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="B379" s="0" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>70</v>
+        <v>469</v>
       </c>
       <c r="D379" s="0">
-        <v>10522</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="0" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B380" s="0" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C380" s="0" t="s">
         <v>70</v>
       </c>
       <c r="D380" s="0">
-        <v>19481</v>
+        <v>10522</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="0" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="B381" s="0" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>819</v>
+        <v>70</v>
       </c>
       <c r="D381" s="0">
-        <v>1080</v>
+        <v>19481</v>
       </c>
     </row>
     <row r="382">
@@ -8655,24 +8664,24 @@
         <v>821</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>18</v>
+        <v>822</v>
       </c>
       <c r="D382" s="0">
-        <v>586.49</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="0" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B383" s="0" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>824</v>
+        <v>18</v>
       </c>
       <c r="D383" s="0">
-        <v>520</v>
+        <v>586.49</v>
       </c>
     </row>
     <row r="384">
@@ -8683,108 +8692,108 @@
         <v>826</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="D384" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="0" t="s">
+        <v>828</v>
+      </c>
+      <c r="B385" s="0" t="s">
+        <v>829</v>
+      </c>
+      <c r="C385" s="0" t="s">
         <v>827</v>
       </c>
-      <c r="B385" s="0" t="s">
-        <v>828</v>
-      </c>
-      <c r="C385" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D385" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="0" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="B386" s="0" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="C386" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D386" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="0" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="B387" s="0" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D387" s="0">
-        <v>5190.9</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="0" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="B388" s="0" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="D388" s="0">
-        <v>2969</v>
+        <v>5190.9</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="0" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="B389" s="0" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D389" s="0">
-        <v>3800</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="0" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="B390" s="0" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D390" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="0" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="B391" s="0" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>841</v>
+        <v>15</v>
       </c>
       <c r="D391" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="392">
@@ -8795,318 +8804,318 @@
         <v>843</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>21</v>
+        <v>844</v>
       </c>
       <c r="D392" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="0" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B393" s="0" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="D393" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="0" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="B394" s="0" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="D394" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="0" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="B395" s="0" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D395" s="0">
-        <v>146.41</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="0" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="B396" s="0" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>207</v>
+        <v>92</v>
       </c>
       <c r="D396" s="0">
-        <v>65537</v>
+        <v>146.41</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="0" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="B397" s="0" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>140</v>
+        <v>207</v>
       </c>
       <c r="D397" s="0">
-        <v>4130.4</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="0" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="B398" s="0" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C398" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D398" s="0">
-        <v>4283</v>
+        <v>4130.4</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="0" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B399" s="0" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="C399" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D399" s="0">
-        <v>6524.8</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="0" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="B400" s="0" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>308</v>
+        <v>140</v>
       </c>
       <c r="D400" s="0">
-        <v>570</v>
+        <v>6524.8</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="0" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="B401" s="0" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>70</v>
+        <v>308</v>
       </c>
       <c r="D401" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="0" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="B402" s="0" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D402" s="0">
-        <v>153</v>
+        <v>550</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="0" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="B403" s="0" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="D403" s="0">
-        <v>740.7</v>
+        <v>153</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="0" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="B404" s="0" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="D404" s="0">
-        <v>101000</v>
+        <v>740.7</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="0" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="B405" s="0" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>123</v>
+        <v>59</v>
       </c>
       <c r="D405" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="0" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="B406" s="0" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="D406" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="0" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="B407" s="0" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D407" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="0" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B408" s="0" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="D408" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="0" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B409" s="0" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="C409" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D409" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="0" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B410" s="0" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="C410" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D410" s="0">
-        <v>2150</v>
+        <v>450</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="0" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="B411" s="0" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>580</v>
+        <v>151</v>
       </c>
       <c r="D411" s="0">
-        <v>25192.82</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="0" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="B412" s="0" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>70</v>
+        <v>580</v>
       </c>
       <c r="D412" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="0" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B413" s="0" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>175</v>
+        <v>70</v>
       </c>
       <c r="D413" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="0" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B414" s="0" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>888</v>
+        <v>175</v>
       </c>
       <c r="D414" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="415">
@@ -9117,189 +9126,189 @@
         <v>890</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>338</v>
+        <v>891</v>
       </c>
       <c r="D415" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="0" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="B416" s="0" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>40</v>
+        <v>338</v>
       </c>
       <c r="D416" s="0">
-        <v>27991.54</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="0" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="B417" s="0" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>140</v>
+        <v>40</v>
       </c>
       <c r="D417" s="0">
-        <v>1020</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="0" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="B418" s="0" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="C418" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D418" s="0">
-        <v>4106</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="0" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="B419" s="0" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>281</v>
+        <v>140</v>
       </c>
       <c r="D419" s="0">
-        <v>450</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="0" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="B420" s="0" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>45</v>
+        <v>281</v>
       </c>
       <c r="D420" s="0">
-        <v>6344.43</v>
+        <v>450</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="0" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="B421" s="0" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="C421" s="0" t="s">
         <v>45</v>
       </c>
       <c r="D421" s="0">
-        <v>2862.28</v>
+        <v>6344.43</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="0" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="B422" s="0" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="C422" s="0" t="s">
         <v>45</v>
       </c>
       <c r="D422" s="0">
-        <v>2131.18</v>
+        <v>2862.28</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="0" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="B423" s="0" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="C423" s="0" t="s">
         <v>45</v>
       </c>
       <c r="D423" s="0">
-        <v>29795.68</v>
+        <v>2131.18</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="0" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="B424" s="0" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="C424" s="0" t="s">
         <v>45</v>
       </c>
       <c r="D424" s="0">
-        <v>2307.09</v>
+        <v>29795.68</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="0" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="B425" s="0" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="C425" s="0" t="s">
         <v>45</v>
       </c>
       <c r="D425" s="0">
-        <v>5249.48</v>
+        <v>2307.09</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="0" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="B426" s="0" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="C426" s="0" t="s">
         <v>45</v>
       </c>
       <c r="D426" s="0">
-        <v>4708</v>
+        <v>5249.48</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="0" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="B427" s="0" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>478</v>
+        <v>45</v>
       </c>
       <c r="D427" s="0">
-        <v>510</v>
+        <v>4708</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="0" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="B428" s="0" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>37</v>
+        <v>478</v>
       </c>
       <c r="D428" s="0">
         <v>510</v>
@@ -9307,16 +9316,16 @@
     </row>
     <row r="429">
       <c r="A429" s="0" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="B429" s="0" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>919</v>
+        <v>37</v>
       </c>
       <c r="D429" s="0">
-        <v>626</v>
+        <v>510</v>
       </c>
     </row>
     <row r="430">
@@ -9327,7 +9336,7 @@
         <v>921</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D430" s="0">
         <v>626</v>
@@ -9335,13 +9344,13 @@
     </row>
     <row r="431">
       <c r="A431" s="0" t="s">
+        <v>923</v>
+      </c>
+      <c r="B431" s="0" t="s">
+        <v>924</v>
+      </c>
+      <c r="C431" s="0" t="s">
         <v>922</v>
-      </c>
-      <c r="B431" s="0" t="s">
-        <v>923</v>
-      </c>
-      <c r="C431" s="0" t="s">
-        <v>919</v>
       </c>
       <c r="D431" s="0">
         <v>626</v>
@@ -9349,27 +9358,27 @@
     </row>
     <row r="432">
       <c r="A432" s="0" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B432" s="0" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D432" s="0">
-        <v>342</v>
+        <v>626</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="0" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="B433" s="0" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D433" s="0">
         <v>342</v>
@@ -9377,13 +9386,13 @@
     </row>
     <row r="434">
       <c r="A434" s="0" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="B434" s="0" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D434" s="0">
         <v>342</v>
@@ -9391,27 +9400,27 @@
     </row>
     <row r="435">
       <c r="A435" s="0" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="B435" s="0" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D435" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="0" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="B436" s="0" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D436" s="0">
         <v>0</v>
@@ -9419,16 +9428,16 @@
     </row>
     <row r="437">
       <c r="A437" s="0" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="B437" s="0" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>936</v>
+        <v>922</v>
       </c>
       <c r="D437" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="438">
@@ -9439,7 +9448,7 @@
         <v>938</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>919</v>
+        <v>939</v>
       </c>
       <c r="D438" s="0">
         <v>453</v>
@@ -9447,41 +9456,41 @@
     </row>
     <row r="439">
       <c r="A439" s="0" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="B439" s="0" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>70</v>
+        <v>922</v>
       </c>
       <c r="D439" s="0">
-        <v>19322</v>
+        <v>453</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="0" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="B440" s="0" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D440" s="0">
-        <v>430</v>
+        <v>19322</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="0" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="B441" s="0" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>281</v>
+        <v>34</v>
       </c>
       <c r="D441" s="0">
         <v>430</v>
@@ -9489,100 +9498,100 @@
     </row>
     <row r="442">
       <c r="A442" s="0" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="B442" s="0" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>115</v>
+        <v>281</v>
       </c>
       <c r="D442" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="0" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="B443" s="0" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="D443" s="0">
-        <v>15400</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="0" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B444" s="0" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="C444" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D444" s="0">
-        <v>3340</v>
+        <v>15400</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="0" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="B445" s="0" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D445" s="0">
-        <v>266200</v>
+        <v>3340</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="0" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B446" s="0" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="C446" s="0" t="s">
         <v>92</v>
       </c>
       <c r="D446" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="0" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B447" s="0" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="C447" s="0" t="s">
         <v>92</v>
       </c>
       <c r="D447" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="0" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B448" s="0" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>959</v>
+        <v>92</v>
       </c>
       <c r="D448" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="449">
@@ -9593,108 +9602,108 @@
         <v>961</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="D449" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="0" t="s">
+        <v>963</v>
+      </c>
+      <c r="B450" s="0" t="s">
+        <v>964</v>
+      </c>
+      <c r="C450" s="0" t="s">
         <v>962</v>
       </c>
-      <c r="B450" s="0" t="s">
-        <v>963</v>
-      </c>
-      <c r="C450" s="0" t="s">
-        <v>959</v>
-      </c>
       <c r="D450" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="0" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B451" s="0" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="D451" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="0" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="B452" s="0" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="D452" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="0" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B453" s="0" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>70</v>
+        <v>962</v>
       </c>
       <c r="D453" s="0">
-        <v>4276</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="0" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="B454" s="0" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="D454" s="0">
-        <v>3930</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="0" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="B455" s="0" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D455" s="0">
-        <v>4392.3</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="0" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B456" s="0" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>976</v>
+        <v>92</v>
       </c>
       <c r="D456" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="457">
@@ -9705,122 +9714,122 @@
         <v>978</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>52</v>
+        <v>979</v>
       </c>
       <c r="D457" s="0">
-        <v>1297</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="0" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="B458" s="0" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="C458" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D458" s="0">
-        <v>298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="0" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="B459" s="0" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="C459" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D459" s="0">
-        <v>596</v>
+        <v>298</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="0" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="B460" s="0" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>376</v>
+        <v>52</v>
       </c>
       <c r="D460" s="0">
-        <v>65142.6</v>
+        <v>596</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="0" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="B461" s="0" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="C461" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D461" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="0" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="B462" s="0" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="D462" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="0" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="B463" s="0" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D463" s="0">
-        <v>12000</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="0" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="B464" s="0" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="C464" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D464" s="0">
-        <v>17425</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="B465" s="0" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>995</v>
+        <v>52</v>
       </c>
       <c r="D465" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="466">
@@ -9834,7 +9843,7 @@
         <v>998</v>
       </c>
       <c r="D466" s="0">
-        <v>2282.3</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="467">
@@ -9848,7 +9857,7 @@
         <v>1001</v>
       </c>
       <c r="D467" s="0">
-        <v>386</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="468">
@@ -9862,7 +9871,7 @@
         <v>1004</v>
       </c>
       <c r="D468" s="0">
-        <v>385.4</v>
+        <v>386</v>
       </c>
     </row>
     <row r="469">
@@ -9873,147 +9882,147 @@
         <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>92</v>
+        <v>1007</v>
       </c>
       <c r="D469" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="0" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B470" s="0" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>123</v>
+        <v>92</v>
       </c>
       <c r="D470" s="0">
-        <v>1890</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="0" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="B471" s="0" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>580</v>
+        <v>123</v>
       </c>
       <c r="D471" s="0">
-        <v>71176.4</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="0" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B472" s="0" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>140</v>
+        <v>580</v>
       </c>
       <c r="D472" s="0">
-        <v>87</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="0" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="B473" s="0" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="D473" s="0">
-        <v>950</v>
+        <v>87</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="0" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="B474" s="0" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>469</v>
+        <v>70</v>
       </c>
       <c r="D474" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="0" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="B475" s="0" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>160</v>
+        <v>469</v>
       </c>
       <c r="D475" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="0" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="B476" s="0" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>478</v>
+        <v>160</v>
       </c>
       <c r="D476" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="0" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="B477" s="0" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>70</v>
+        <v>478</v>
       </c>
       <c r="D477" s="0">
-        <v>5790</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="0" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="B478" s="0" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>919</v>
+        <v>70</v>
       </c>
       <c r="D478" s="0">
-        <v>880</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="0" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="B479" s="0" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D479" s="0">
         <v>880</v>
@@ -10021,13 +10030,13 @@
     </row>
     <row r="480">
       <c r="A480" s="0" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B480" s="0" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="D480" s="0">
         <v>880</v>
@@ -10035,114 +10044,114 @@
     </row>
     <row r="481">
       <c r="A481" s="0" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="B481" s="0" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>21</v>
+        <v>922</v>
       </c>
       <c r="D481" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="0" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="B482" s="0" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D482" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="0" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="B483" s="0" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="C483" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D483" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="B484" s="0" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D484" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B485" s="0" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C485" s="0" t="s">
         <v>281</v>
       </c>
       <c r="D485" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="0" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="B486" s="0" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D486" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="0" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B487" s="0" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="C487" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D487" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="0" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="B488" s="0" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>1045</v>
+        <v>15</v>
       </c>
       <c r="D488" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="489">
@@ -10153,94 +10162,94 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>28</v>
+        <v>1048</v>
       </c>
       <c r="D489" s="0">
-        <v>15189</v>
+        <v>1</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="0" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B490" s="0" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>376</v>
+        <v>28</v>
       </c>
       <c r="D490" s="0">
-        <v>3859.93</v>
+        <v>15189</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="0" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="B491" s="0" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="C491" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D491" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="0" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="B492" s="0" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D492" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="0" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="B493" s="0" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="C493" s="0" t="s">
         <v>338</v>
       </c>
       <c r="D493" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="0" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="B494" s="0" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>37</v>
+        <v>338</v>
       </c>
       <c r="D494" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="0" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="B495" s="0" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>1060</v>
+        <v>37</v>
       </c>
       <c r="D495" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="496">
@@ -10251,191 +10260,205 @@
         <v>1062</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>105</v>
+        <v>1063</v>
       </c>
       <c r="D496" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="0" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="B497" s="0" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D497" s="0">
-        <v>43590.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="0" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="B498" s="0" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="C498" s="0" t="s">
-        <v>469</v>
+        <v>92</v>
       </c>
       <c r="D498" s="0">
-        <v>207558.07</v>
+        <v>43590.25</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="0" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="B499" s="0" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="C499" s="0" t="s">
-        <v>376</v>
+        <v>469</v>
       </c>
       <c r="D499" s="0">
-        <v>77429.29</v>
+        <v>207558.07</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="0" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="B500" s="0" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="C500" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D500" s="0">
-        <v>42913.42</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="0" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="B501" s="0" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="C501" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D501" s="0">
-        <v>88806.25</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="0" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="B502" s="0" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="C502" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D502" s="0">
-        <v>50781.52</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="0" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="B503" s="0" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="C503" s="0" t="s">
-        <v>21</v>
+        <v>376</v>
       </c>
       <c r="D503" s="0">
-        <v>1600</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="0" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="B504" s="0" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="C504" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D504" s="0">
-        <v>3521.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="0" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="B505" s="0" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="C505" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D505" s="0">
-        <v>3987</v>
+        <v>3521.4</v>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="0" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="B506" s="0" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="C506" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D506" s="0">
-        <v>4086.37</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="0" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="B507" s="0" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="C507" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D507" s="0">
-        <v>3382.65</v>
+        <v>4086.37</v>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="0" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="B508" s="0" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="C508" s="0" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="D508" s="0">
-        <v>430</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="B509" s="0" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="C509" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D509" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="0" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B510" s="0" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C510" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="D509" s="0">
+      <c r="D510" s="0">
         <v>465</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb 26/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -4151,7 +4151,7 @@
         <v>140</v>
       </c>
       <c r="D59" s="0">
-        <v>489.8</v>
+        <v>500</v>
       </c>
     </row>
     <row r="60">
@@ -4333,7 +4333,7 @@
         <v>140</v>
       </c>
       <c r="D72" s="0">
-        <v>649</v>
+        <v>700</v>
       </c>
     </row>
     <row r="73">
@@ -4935,7 +4935,7 @@
         <v>140</v>
       </c>
       <c r="D115" s="0">
-        <v>993</v>
+        <v>970</v>
       </c>
     </row>
     <row r="116">
@@ -5159,7 +5159,7 @@
         <v>140</v>
       </c>
       <c r="D131" s="0">
-        <v>2800</v>
+        <v>3100</v>
       </c>
     </row>
     <row r="132">
@@ -5173,7 +5173,7 @@
         <v>140</v>
       </c>
       <c r="D132" s="0">
-        <v>6536</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="133">
@@ -6307,7 +6307,7 @@
         <v>472</v>
       </c>
       <c r="D213" s="0">
-        <v>60630</v>
+        <v>70443</v>
       </c>
     </row>
     <row r="214">
@@ -6965,7 +6965,7 @@
         <v>140</v>
       </c>
       <c r="D260" s="0">
-        <v>430</v>
+        <v>446</v>
       </c>
     </row>
     <row r="261">
@@ -6979,7 +6979,7 @@
         <v>140</v>
       </c>
       <c r="D261" s="0">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="262">
@@ -7049,7 +7049,7 @@
         <v>582</v>
       </c>
       <c r="D266" s="0">
-        <v>177940.1</v>
+        <v>189016.25</v>
       </c>
     </row>
     <row r="267">
@@ -7091,7 +7091,7 @@
         <v>472</v>
       </c>
       <c r="D269" s="0">
-        <v>227939.52</v>
+        <v>243315</v>
       </c>
     </row>
     <row r="270">
@@ -7105,7 +7105,7 @@
         <v>472</v>
       </c>
       <c r="D270" s="0">
-        <v>184488.7</v>
+        <v>196835</v>
       </c>
     </row>
     <row r="271">
@@ -7497,7 +7497,7 @@
         <v>140</v>
       </c>
       <c r="D298" s="0">
-        <v>4590</v>
+        <v>4730</v>
       </c>
     </row>
     <row r="299">
@@ -7511,7 +7511,7 @@
         <v>140</v>
       </c>
       <c r="D299" s="0">
-        <v>2300</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="300">
@@ -7525,7 +7525,7 @@
         <v>140</v>
       </c>
       <c r="D300" s="0">
-        <v>1150</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="301">
@@ -7693,7 +7693,7 @@
         <v>140</v>
       </c>
       <c r="D312" s="0">
-        <v>1250</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="313">
@@ -7987,7 +7987,7 @@
         <v>140</v>
       </c>
       <c r="D333" s="0">
-        <v>890</v>
+        <v>935</v>
       </c>
     </row>
     <row r="334">
@@ -8001,7 +8001,7 @@
         <v>140</v>
       </c>
       <c r="D334" s="0">
-        <v>594</v>
+        <v>620</v>
       </c>
     </row>
     <row r="335">
@@ -8015,7 +8015,7 @@
         <v>140</v>
       </c>
       <c r="D335" s="0">
-        <v>65</v>
+        <v>73</v>
       </c>
     </row>
     <row r="336">
@@ -8323,7 +8323,7 @@
         <v>140</v>
       </c>
       <c r="D357" s="0">
-        <v>350</v>
+        <v>365</v>
       </c>
     </row>
     <row r="358">
@@ -8631,7 +8631,7 @@
         <v>472</v>
       </c>
       <c r="D379" s="0">
-        <v>207558.08</v>
+        <v>213700</v>
       </c>
     </row>
     <row r="380">
@@ -8645,7 +8645,7 @@
         <v>472</v>
       </c>
       <c r="D380" s="0">
-        <v>249069.69</v>
+        <v>257000</v>
       </c>
     </row>
     <row r="381">
@@ -9037,7 +9037,7 @@
         <v>140</v>
       </c>
       <c r="D408" s="0">
-        <v>857.67</v>
+        <v>883</v>
       </c>
     </row>
     <row r="409">
@@ -9555,7 +9555,7 @@
         <v>140</v>
       </c>
       <c r="D445" s="0">
-        <v>15400</v>
+        <v>12049</v>
       </c>
     </row>
     <row r="446">
@@ -9569,7 +9569,7 @@
         <v>140</v>
       </c>
       <c r="D446" s="0">
-        <v>3340</v>
+        <v>2895</v>
       </c>
     </row>
     <row r="447">
@@ -9947,7 +9947,7 @@
         <v>582</v>
       </c>
       <c r="D473" s="0">
-        <v>71176.4</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="474">
@@ -9961,7 +9961,7 @@
         <v>140</v>
       </c>
       <c r="D474" s="0">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="475">
@@ -9989,7 +9989,7 @@
         <v>472</v>
       </c>
       <c r="D476" s="0">
-        <v>342641</v>
+        <v>398107</v>
       </c>
     </row>
     <row r="477">
@@ -10325,7 +10325,7 @@
         <v>472</v>
       </c>
       <c r="D500" s="0">
-        <v>207558.07</v>
+        <v>213700</v>
       </c>
     </row>
     <row r="501">
@@ -10479,7 +10479,7 @@
         <v>140</v>
       </c>
       <c r="D511" s="0">
-        <v>465</v>
+        <v>495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync: stock y precios actualizados mié 30/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3591,7 +3591,7 @@
         <v>45</v>
       </c>
       <c r="D19" s="0">
-        <v>3853.39</v>
+        <v>3958.98</v>
       </c>
     </row>
     <row r="20">
@@ -3619,7 +3619,7 @@
         <v>45</v>
       </c>
       <c r="D21" s="0">
-        <v>31996.8</v>
+        <v>32755.59</v>
       </c>
     </row>
     <row r="22">
@@ -4907,7 +4907,7 @@
         <v>45</v>
       </c>
       <c r="D113" s="0">
-        <v>5771.79</v>
+        <v>5660.43</v>
       </c>
     </row>
     <row r="114">
@@ -6125,7 +6125,7 @@
         <v>45</v>
       </c>
       <c r="D200" s="0">
-        <v>4729.48</v>
+        <v>6127.17</v>
       </c>
     </row>
     <row r="201">
@@ -8085,7 +8085,7 @@
         <v>45</v>
       </c>
       <c r="D340" s="0">
-        <v>5780.66</v>
+        <v>5726.32</v>
       </c>
     </row>
     <row r="341">
@@ -9233,7 +9233,7 @@
         <v>45</v>
       </c>
       <c r="D422" s="0">
-        <v>6344.43</v>
+        <v>6518.32</v>
       </c>
     </row>
     <row r="423">
@@ -9247,7 +9247,7 @@
         <v>45</v>
       </c>
       <c r="D423" s="0">
-        <v>2862.28</v>
+        <v>2940.72</v>
       </c>
     </row>
     <row r="424">
@@ -9261,7 +9261,7 @@
         <v>45</v>
       </c>
       <c r="D424" s="0">
-        <v>2131.18</v>
+        <v>2090.06</v>
       </c>
     </row>
     <row r="425">
@@ -9275,7 +9275,7 @@
         <v>45</v>
       </c>
       <c r="D425" s="0">
-        <v>29795.68</v>
+        <v>30612.7</v>
       </c>
     </row>
     <row r="426">
@@ -9289,7 +9289,7 @@
         <v>45</v>
       </c>
       <c r="D426" s="0">
-        <v>2307.09</v>
+        <v>2370.33</v>
       </c>
     </row>
     <row r="427">
@@ -9303,7 +9303,7 @@
         <v>45</v>
       </c>
       <c r="D427" s="0">
-        <v>5249.48</v>
+        <v>6550.3</v>
       </c>
     </row>
     <row r="428">
@@ -9317,7 +9317,7 @@
         <v>45</v>
       </c>
       <c r="D428" s="0">
-        <v>4708</v>
+        <v>5277.18</v>
       </c>
     </row>
     <row r="429">

</xml_diff>

<commit_message>
sync: stock y precios actualizados jue 01/10/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -5383,7 +5383,7 @@
         <v>31</v>
       </c>
       <c r="D147" s="0">
-        <v>700</v>
+        <v>550</v>
       </c>
     </row>
     <row r="148">
@@ -5397,7 +5397,7 @@
         <v>70</v>
       </c>
       <c r="D148" s="0">
-        <v>700</v>
+        <v>550</v>
       </c>
     </row>
     <row r="149">
@@ -5411,7 +5411,7 @@
         <v>34</v>
       </c>
       <c r="D149" s="0">
-        <v>700</v>
+        <v>550</v>
       </c>
     </row>
     <row r="150">
@@ -5481,7 +5481,7 @@
         <v>34</v>
       </c>
       <c r="D154" s="0">
-        <v>400</v>
+        <v>380</v>
       </c>
     </row>
     <row r="155">
@@ -5495,7 +5495,7 @@
         <v>70</v>
       </c>
       <c r="D155" s="0">
-        <v>410</v>
+        <v>380</v>
       </c>
     </row>
     <row r="156">
@@ -5607,7 +5607,7 @@
         <v>34</v>
       </c>
       <c r="D163" s="0">
-        <v>650</v>
+        <v>550</v>
       </c>
     </row>
     <row r="164">
@@ -5621,7 +5621,7 @@
         <v>151</v>
       </c>
       <c r="D164" s="0">
-        <v>650</v>
+        <v>550</v>
       </c>
     </row>
     <row r="165">
@@ -5635,7 +5635,7 @@
         <v>15</v>
       </c>
       <c r="D165" s="0">
-        <v>650</v>
+        <v>550</v>
       </c>
     </row>
     <row r="166">
@@ -8043,7 +8043,7 @@
         <v>34</v>
       </c>
       <c r="D337" s="0">
-        <v>420</v>
+        <v>400</v>
       </c>
     </row>
     <row r="338">
@@ -8057,7 +8057,7 @@
         <v>362</v>
       </c>
       <c r="D338" s="0">
-        <v>418</v>
+        <v>400</v>
       </c>
     </row>
     <row r="339">

</xml_diff>

<commit_message>
sync: stock y precios actualizados mar 06/10/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3669,7 +3669,7 @@
         <v>45</v>
       </c>
       <c r="D19" s="0">
-        <v>3958.98</v>
+        <v>3886.27</v>
       </c>
     </row>
     <row r="20">
@@ -3697,7 +3697,7 @@
         <v>45</v>
       </c>
       <c r="D21" s="0">
-        <v>32755.59</v>
+        <v>32153.98</v>
       </c>
     </row>
     <row r="22">
@@ -5013,7 +5013,7 @@
         <v>45</v>
       </c>
       <c r="D115" s="0">
-        <v>5660.43</v>
+        <v>5556.47</v>
       </c>
     </row>
     <row r="116">
@@ -6231,7 +6231,7 @@
         <v>45</v>
       </c>
       <c r="D202" s="0">
-        <v>6127.17</v>
+        <v>6014.63</v>
       </c>
     </row>
     <row r="203">
@@ -8331,7 +8331,7 @@
         <v>45</v>
       </c>
       <c r="D352" s="0">
-        <v>5726.32</v>
+        <v>5621.15</v>
       </c>
     </row>
     <row r="353">
@@ -9493,7 +9493,7 @@
         <v>45</v>
       </c>
       <c r="D435" s="0">
-        <v>6518.32</v>
+        <v>6398.6</v>
       </c>
     </row>
     <row r="436">
@@ -9507,7 +9507,7 @@
         <v>45</v>
       </c>
       <c r="D436" s="0">
-        <v>2940.72</v>
+        <v>2886.7</v>
       </c>
     </row>
     <row r="437">
@@ -9521,7 +9521,7 @@
         <v>45</v>
       </c>
       <c r="D437" s="0">
-        <v>2090.06</v>
+        <v>2050.95</v>
       </c>
     </row>
     <row r="438">
@@ -9535,7 +9535,7 @@
         <v>45</v>
       </c>
       <c r="D438" s="0">
-        <v>30612.7</v>
+        <v>30050.45</v>
       </c>
     </row>
     <row r="439">
@@ -9549,7 +9549,7 @@
         <v>45</v>
       </c>
       <c r="D439" s="0">
-        <v>2370.33</v>
+        <v>2326.8</v>
       </c>
     </row>
     <row r="440">
@@ -9563,7 +9563,7 @@
         <v>45</v>
       </c>
       <c r="D440" s="0">
-        <v>6550.3</v>
+        <v>6429.95</v>
       </c>
     </row>
     <row r="441">
@@ -9577,7 +9577,7 @@
         <v>45</v>
       </c>
       <c r="D441" s="0">
-        <v>5277.18</v>
+        <v>5180.26</v>
       </c>
     </row>
     <row r="442">

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb 10/10/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3977,7 +3977,7 @@
         <v>97</v>
       </c>
       <c r="D41" s="0">
-        <v>22627</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="42">
@@ -4173,7 +4173,7 @@
         <v>97</v>
       </c>
       <c r="D55" s="0">
-        <v>35271.5</v>
+        <v>36602.5</v>
       </c>
     </row>
     <row r="56">
@@ -7953,7 +7953,7 @@
         <v>97</v>
       </c>
       <c r="D325" s="0">
-        <v>332750</v>
+        <v>342732.5</v>
       </c>
     </row>
     <row r="326">
@@ -8051,7 +8051,7 @@
         <v>97</v>
       </c>
       <c r="D332" s="0">
-        <v>25289</v>
+        <v>26620</v>
       </c>
     </row>
     <row r="333">
@@ -8065,7 +8065,7 @@
         <v>97</v>
       </c>
       <c r="D333" s="0">
-        <v>252890</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="334">

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb 17/10/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="1120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="1122">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -1293,6 +1293,12 @@
   </si>
   <si>
     <t>FABOGESIC DICLO 75MG X 15 COMPR - 000024490</t>
+  </si>
+  <si>
+    <t>000024722</t>
+  </si>
+  <si>
+    <t>FABOGESIC PLEN 50/4MG X 10 COMPR - RELAX - SAVANT - 000024722</t>
   </si>
   <si>
     <t>000024436</t>
@@ -3437,7 +3443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D524"/>
+  <dimension ref="A2:D525"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -6091,7 +6097,7 @@
         <v>18</v>
       </c>
       <c r="D192" s="0">
-        <v>2184.81</v>
+        <v>320</v>
       </c>
     </row>
     <row r="193">
@@ -6102,10 +6108,10 @@
         <v>430</v>
       </c>
       <c r="C193" s="0" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D193" s="0">
-        <v>9748.5</v>
+        <v>2184.81</v>
       </c>
     </row>
     <row r="194">
@@ -6116,10 +6122,10 @@
         <v>432</v>
       </c>
       <c r="C194" s="0" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="D194" s="0">
-        <v>430</v>
+        <v>9748.5</v>
       </c>
     </row>
     <row r="195">
@@ -6133,7 +6139,7 @@
         <v>75</v>
       </c>
       <c r="D195" s="0">
-        <v>800</v>
+        <v>430</v>
       </c>
     </row>
     <row r="196">
@@ -6144,10 +6150,10 @@
         <v>436</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>250</v>
+        <v>75</v>
       </c>
       <c r="D196" s="0">
-        <v>2040</v>
+        <v>800</v>
       </c>
     </row>
     <row r="197">
@@ -6161,7 +6167,7 @@
         <v>250</v>
       </c>
       <c r="D197" s="0">
-        <v>1380</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="198">
@@ -6172,10 +6178,10 @@
         <v>440</v>
       </c>
       <c r="C198" s="0" t="s">
-        <v>384</v>
+        <v>250</v>
       </c>
       <c r="D198" s="0">
-        <v>236458.17</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="199">
@@ -6186,10 +6192,10 @@
         <v>442</v>
       </c>
       <c r="C199" s="0" t="s">
-        <v>28</v>
+        <v>384</v>
       </c>
       <c r="D199" s="0">
-        <v>317.2</v>
+        <v>236458.17</v>
       </c>
     </row>
     <row r="200">
@@ -6200,10 +6206,10 @@
         <v>444</v>
       </c>
       <c r="C200" s="0" t="s">
-        <v>384</v>
+        <v>28</v>
       </c>
       <c r="D200" s="0">
-        <v>25100</v>
+        <v>317.2</v>
       </c>
     </row>
     <row r="201">
@@ -6214,24 +6220,24 @@
         <v>446</v>
       </c>
       <c r="C201" s="0" t="s">
-        <v>447</v>
+        <v>384</v>
       </c>
       <c r="D201" s="0">
-        <v>20900</v>
+        <v>25100</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="0" t="s">
+        <v>447</v>
+      </c>
+      <c r="B202" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="B202" s="0" t="s">
+      <c r="C202" s="0" t="s">
         <v>449</v>
       </c>
-      <c r="C202" s="0" t="s">
-        <v>45</v>
-      </c>
       <c r="D202" s="0">
-        <v>6014.63</v>
+        <v>20900</v>
       </c>
     </row>
     <row r="203">
@@ -6242,10 +6248,10 @@
         <v>451</v>
       </c>
       <c r="C203" s="0" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D203" s="0">
-        <v>1104.46</v>
+        <v>6014.63</v>
       </c>
     </row>
     <row r="204">
@@ -6256,10 +6262,10 @@
         <v>453</v>
       </c>
       <c r="C204" s="0" t="s">
-        <v>97</v>
+        <v>21</v>
       </c>
       <c r="D204" s="0">
-        <v>11646.25</v>
+        <v>1104.46</v>
       </c>
     </row>
     <row r="205">
@@ -6270,10 +6276,10 @@
         <v>455</v>
       </c>
       <c r="C205" s="0" t="s">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="D205" s="0">
-        <v>6072</v>
+        <v>11646.25</v>
       </c>
     </row>
     <row r="206">
@@ -6284,10 +6290,10 @@
         <v>457</v>
       </c>
       <c r="C206" s="0" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="D206" s="0">
-        <v>400</v>
+        <v>6072</v>
       </c>
     </row>
     <row r="207">
@@ -6298,10 +6304,10 @@
         <v>459</v>
       </c>
       <c r="C207" s="0" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="D207" s="0">
-        <v>409</v>
+        <v>400</v>
       </c>
     </row>
     <row r="208">
@@ -6312,10 +6318,10 @@
         <v>461</v>
       </c>
       <c r="C208" s="0" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="D208" s="0">
-        <v>10748</v>
+        <v>409</v>
       </c>
     </row>
     <row r="209">
@@ -6329,7 +6335,7 @@
         <v>69</v>
       </c>
       <c r="D209" s="0">
-        <v>12898</v>
+        <v>10748</v>
       </c>
     </row>
     <row r="210">
@@ -6340,10 +6346,10 @@
         <v>465</v>
       </c>
       <c r="C210" s="0" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="D210" s="0">
-        <v>2000</v>
+        <v>12898</v>
       </c>
     </row>
     <row r="211">
@@ -6354,24 +6360,24 @@
         <v>467</v>
       </c>
       <c r="C211" s="0" t="s">
-        <v>468</v>
+        <v>52</v>
       </c>
       <c r="D211" s="0">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="0" t="s">
+        <v>468</v>
+      </c>
+      <c r="B212" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="B212" s="0" t="s">
+      <c r="C212" s="0" t="s">
         <v>470</v>
       </c>
-      <c r="C212" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D212" s="0">
-        <v>490</v>
+        <v>0</v>
       </c>
     </row>
     <row r="213">
@@ -6382,10 +6388,10 @@
         <v>472</v>
       </c>
       <c r="C213" s="0" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D213" s="0">
-        <v>0</v>
+        <v>490</v>
       </c>
     </row>
     <row r="214">
@@ -6396,10 +6402,10 @@
         <v>474</v>
       </c>
       <c r="C214" s="0" t="s">
-        <v>165</v>
+        <v>34</v>
       </c>
       <c r="D214" s="0">
-        <v>25171.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="215">
@@ -6410,24 +6416,24 @@
         <v>476</v>
       </c>
       <c r="C215" s="0" t="s">
-        <v>477</v>
+        <v>165</v>
       </c>
       <c r="D215" s="0">
-        <v>70443</v>
+        <v>25171.1</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="s">
+        <v>477</v>
+      </c>
+      <c r="B216" s="0" t="s">
         <v>478</v>
       </c>
-      <c r="B216" s="0" t="s">
+      <c r="C216" s="0" t="s">
         <v>479</v>
       </c>
-      <c r="C216" s="0" t="s">
-        <v>156</v>
-      </c>
       <c r="D216" s="0">
-        <v>1800</v>
+        <v>70443</v>
       </c>
     </row>
     <row r="217">
@@ -6438,10 +6444,10 @@
         <v>481</v>
       </c>
       <c r="C217" s="0" t="s">
-        <v>34</v>
+        <v>156</v>
       </c>
       <c r="D217" s="0">
-        <v>0</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="218">
@@ -6452,10 +6458,10 @@
         <v>483</v>
       </c>
       <c r="C218" s="0" t="s">
-        <v>145</v>
+        <v>34</v>
       </c>
       <c r="D218" s="0">
-        <v>492.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="219">
@@ -6466,10 +6472,10 @@
         <v>485</v>
       </c>
       <c r="C219" s="0" t="s">
-        <v>212</v>
+        <v>145</v>
       </c>
       <c r="D219" s="0">
-        <v>495</v>
+        <v>492.2</v>
       </c>
     </row>
     <row r="220">
@@ -6480,10 +6486,10 @@
         <v>487</v>
       </c>
       <c r="C220" s="0" t="s">
-        <v>18</v>
+        <v>212</v>
       </c>
       <c r="D220" s="0">
-        <v>1819.72</v>
+        <v>495</v>
       </c>
     </row>
     <row r="221">
@@ -6497,7 +6503,7 @@
         <v>18</v>
       </c>
       <c r="D221" s="0">
-        <v>4391.81</v>
+        <v>1819.72</v>
       </c>
     </row>
     <row r="222">
@@ -6508,21 +6514,21 @@
         <v>491</v>
       </c>
       <c r="C222" s="0" t="s">
-        <v>492</v>
+        <v>18</v>
       </c>
       <c r="D222" s="0">
-        <v>4100</v>
+        <v>4391.81</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0" t="s">
+        <v>492</v>
+      </c>
+      <c r="B223" s="0" t="s">
         <v>493</v>
       </c>
-      <c r="B223" s="0" t="s">
+      <c r="C223" s="0" t="s">
         <v>494</v>
-      </c>
-      <c r="C223" s="0" t="s">
-        <v>492</v>
       </c>
       <c r="D223" s="0">
         <v>4100</v>
@@ -6536,7 +6542,7 @@
         <v>496</v>
       </c>
       <c r="C224" s="0" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D224" s="0">
         <v>4100</v>
@@ -6550,10 +6556,10 @@
         <v>498</v>
       </c>
       <c r="C225" s="0" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D225" s="0">
-        <v>4200</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="226">
@@ -6564,10 +6570,10 @@
         <v>500</v>
       </c>
       <c r="C226" s="0" t="s">
-        <v>52</v>
+        <v>494</v>
       </c>
       <c r="D226" s="0">
-        <v>4700</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="227">
@@ -6578,10 +6584,10 @@
         <v>502</v>
       </c>
       <c r="C227" s="0" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D227" s="0">
-        <v>235</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="228">
@@ -6620,10 +6626,10 @@
         <v>508</v>
       </c>
       <c r="C230" s="0" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D230" s="0">
-        <v>4670</v>
+        <v>235</v>
       </c>
     </row>
     <row r="231">
@@ -6662,21 +6668,21 @@
         <v>514</v>
       </c>
       <c r="C233" s="0" t="s">
-        <v>515</v>
+        <v>52</v>
       </c>
       <c r="D233" s="0">
-        <v>265</v>
+        <v>4670</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="0" t="s">
+        <v>515</v>
+      </c>
+      <c r="B234" s="0" t="s">
         <v>516</v>
       </c>
-      <c r="B234" s="0" t="s">
+      <c r="C234" s="0" t="s">
         <v>517</v>
-      </c>
-      <c r="C234" s="0" t="s">
-        <v>515</v>
       </c>
       <c r="D234" s="0">
         <v>265</v>
@@ -6690,7 +6696,7 @@
         <v>519</v>
       </c>
       <c r="C235" s="0" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D235" s="0">
         <v>265</v>
@@ -6704,7 +6710,7 @@
         <v>521</v>
       </c>
       <c r="C236" s="0" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D236" s="0">
         <v>265</v>
@@ -6718,7 +6724,7 @@
         <v>523</v>
       </c>
       <c r="C237" s="0" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D237" s="0">
         <v>265</v>
@@ -6732,7 +6738,7 @@
         <v>525</v>
       </c>
       <c r="C238" s="0" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D238" s="0">
         <v>265</v>
@@ -6746,21 +6752,21 @@
         <v>527</v>
       </c>
       <c r="C239" s="0" t="s">
-        <v>528</v>
+        <v>517</v>
       </c>
       <c r="D239" s="0">
-        <v>4700</v>
+        <v>265</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="0" t="s">
+        <v>528</v>
+      </c>
+      <c r="B240" s="0" t="s">
         <v>529</v>
       </c>
-      <c r="B240" s="0" t="s">
+      <c r="C240" s="0" t="s">
         <v>530</v>
-      </c>
-      <c r="C240" s="0" t="s">
-        <v>531</v>
       </c>
       <c r="D240" s="0">
         <v>4700</v>
@@ -6768,13 +6774,13 @@
     </row>
     <row r="241">
       <c r="A241" s="0" t="s">
+        <v>531</v>
+      </c>
+      <c r="B241" s="0" t="s">
         <v>532</v>
       </c>
-      <c r="B241" s="0" t="s">
+      <c r="C241" s="0" t="s">
         <v>533</v>
-      </c>
-      <c r="C241" s="0" t="s">
-        <v>52</v>
       </c>
       <c r="D241" s="0">
         <v>4700</v>
@@ -6791,7 +6797,7 @@
         <v>52</v>
       </c>
       <c r="D242" s="0">
-        <v>597</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="243">
@@ -6805,7 +6811,7 @@
         <v>52</v>
       </c>
       <c r="D243" s="0">
-        <v>223</v>
+        <v>597</v>
       </c>
     </row>
     <row r="244">
@@ -6819,7 +6825,7 @@
         <v>52</v>
       </c>
       <c r="D244" s="0">
-        <v>247</v>
+        <v>223</v>
       </c>
     </row>
     <row r="245">
@@ -6830,10 +6836,10 @@
         <v>541</v>
       </c>
       <c r="C245" s="0" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="D245" s="0">
-        <v>5600</v>
+        <v>247</v>
       </c>
     </row>
     <row r="246">
@@ -6844,10 +6850,10 @@
         <v>543</v>
       </c>
       <c r="C246" s="0" t="s">
-        <v>156</v>
+        <v>37</v>
       </c>
       <c r="D246" s="0">
-        <v>6000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="247">
@@ -6858,10 +6864,10 @@
         <v>545</v>
       </c>
       <c r="C247" s="0" t="s">
-        <v>75</v>
+        <v>156</v>
       </c>
       <c r="D247" s="0">
-        <v>80000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="248">
@@ -6875,7 +6881,7 @@
         <v>75</v>
       </c>
       <c r="D248" s="0">
-        <v>90000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="249">
@@ -6889,7 +6895,7 @@
         <v>75</v>
       </c>
       <c r="D249" s="0">
-        <v>110000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="250">
@@ -6900,10 +6906,10 @@
         <v>551</v>
       </c>
       <c r="C250" s="0" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D250" s="0">
-        <v>900</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="251">
@@ -6914,10 +6920,10 @@
         <v>553</v>
       </c>
       <c r="C251" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D251" s="0">
-        <v>1100</v>
+        <v>900</v>
       </c>
     </row>
     <row r="252">
@@ -6931,7 +6937,7 @@
         <v>15</v>
       </c>
       <c r="D252" s="0">
-        <v>2500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="253">
@@ -6942,10 +6948,10 @@
         <v>557</v>
       </c>
       <c r="C253" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D253" s="0">
-        <v>14608.16</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="254">
@@ -6956,10 +6962,10 @@
         <v>559</v>
       </c>
       <c r="C254" s="0" t="s">
-        <v>156</v>
+        <v>28</v>
       </c>
       <c r="D254" s="0">
-        <v>700</v>
+        <v>14608.16</v>
       </c>
     </row>
     <row r="255">
@@ -6970,7 +6976,7 @@
         <v>561</v>
       </c>
       <c r="C255" s="0" t="s">
-        <v>37</v>
+        <v>156</v>
       </c>
       <c r="D255" s="0">
         <v>700</v>
@@ -6984,10 +6990,10 @@
         <v>563</v>
       </c>
       <c r="C256" s="0" t="s">
-        <v>289</v>
+        <v>37</v>
       </c>
       <c r="D256" s="0">
-        <v>450</v>
+        <v>700</v>
       </c>
     </row>
     <row r="257">
@@ -6998,10 +7004,10 @@
         <v>565</v>
       </c>
       <c r="C257" s="0" t="s">
-        <v>15</v>
+        <v>289</v>
       </c>
       <c r="D257" s="0">
-        <v>555</v>
+        <v>450</v>
       </c>
     </row>
     <row r="258">
@@ -7015,7 +7021,7 @@
         <v>15</v>
       </c>
       <c r="D258" s="0">
-        <v>825</v>
+        <v>555</v>
       </c>
     </row>
     <row r="259">
@@ -7029,7 +7035,7 @@
         <v>15</v>
       </c>
       <c r="D259" s="0">
-        <v>36.3</v>
+        <v>825</v>
       </c>
     </row>
     <row r="260">
@@ -7043,7 +7049,7 @@
         <v>15</v>
       </c>
       <c r="D260" s="0">
-        <v>544.5</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="261">
@@ -7057,7 +7063,7 @@
         <v>15</v>
       </c>
       <c r="D261" s="0">
-        <v>750</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="262">
@@ -7068,10 +7074,10 @@
         <v>575</v>
       </c>
       <c r="C262" s="0" t="s">
-        <v>156</v>
+        <v>15</v>
       </c>
       <c r="D262" s="0">
-        <v>1130</v>
+        <v>750</v>
       </c>
     </row>
     <row r="263">
@@ -7082,10 +7088,10 @@
         <v>577</v>
       </c>
       <c r="C263" s="0" t="s">
-        <v>52</v>
+        <v>156</v>
       </c>
       <c r="D263" s="0">
-        <v>4510</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="264">
@@ -7138,10 +7144,10 @@
         <v>585</v>
       </c>
       <c r="C267" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D267" s="0">
-        <v>902</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="268">
@@ -7155,7 +7161,7 @@
         <v>15</v>
       </c>
       <c r="D268" s="0">
-        <v>880</v>
+        <v>902</v>
       </c>
     </row>
     <row r="269">
@@ -7166,10 +7172,10 @@
         <v>589</v>
       </c>
       <c r="C269" s="0" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="D269" s="0">
-        <v>446</v>
+        <v>880</v>
       </c>
     </row>
     <row r="270">
@@ -7183,7 +7189,7 @@
         <v>145</v>
       </c>
       <c r="D270" s="0">
-        <v>370</v>
+        <v>446</v>
       </c>
     </row>
     <row r="271">
@@ -7194,10 +7200,10 @@
         <v>593</v>
       </c>
       <c r="C271" s="0" t="s">
-        <v>18</v>
+        <v>145</v>
       </c>
       <c r="D271" s="0">
-        <v>300</v>
+        <v>370</v>
       </c>
     </row>
     <row r="272">
@@ -7211,7 +7217,7 @@
         <v>18</v>
       </c>
       <c r="D272" s="0">
-        <v>420</v>
+        <v>300</v>
       </c>
     </row>
     <row r="273">
@@ -7225,7 +7231,7 @@
         <v>18</v>
       </c>
       <c r="D273" s="0">
-        <v>760</v>
+        <v>420</v>
       </c>
     </row>
     <row r="274">
@@ -7239,7 +7245,7 @@
         <v>18</v>
       </c>
       <c r="D274" s="0">
-        <v>820</v>
+        <v>760</v>
       </c>
     </row>
     <row r="275">
@@ -7250,24 +7256,24 @@
         <v>601</v>
       </c>
       <c r="C275" s="0" t="s">
-        <v>602</v>
+        <v>18</v>
       </c>
       <c r="D275" s="0">
-        <v>189016.25</v>
+        <v>820</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="0" t="s">
+        <v>602</v>
+      </c>
+      <c r="B276" s="0" t="s">
         <v>603</v>
       </c>
-      <c r="B276" s="0" t="s">
+      <c r="C276" s="0" t="s">
         <v>604</v>
       </c>
-      <c r="C276" s="0" t="s">
-        <v>75</v>
-      </c>
       <c r="D276" s="0">
-        <v>28000</v>
+        <v>189016.25</v>
       </c>
     </row>
     <row r="277">
@@ -7281,7 +7287,7 @@
         <v>75</v>
       </c>
       <c r="D277" s="0">
-        <v>34000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="278">
@@ -7292,10 +7298,10 @@
         <v>608</v>
       </c>
       <c r="C278" s="0" t="s">
-        <v>477</v>
+        <v>75</v>
       </c>
       <c r="D278" s="0">
-        <v>243315</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="279">
@@ -7306,10 +7312,10 @@
         <v>610</v>
       </c>
       <c r="C279" s="0" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D279" s="0">
-        <v>196835</v>
+        <v>243315</v>
       </c>
     </row>
     <row r="280">
@@ -7320,10 +7326,10 @@
         <v>612</v>
       </c>
       <c r="C280" s="0" t="s">
-        <v>15</v>
+        <v>479</v>
       </c>
       <c r="D280" s="0">
-        <v>1760</v>
+        <v>196835</v>
       </c>
     </row>
     <row r="281">
@@ -7334,24 +7340,24 @@
         <v>614</v>
       </c>
       <c r="C281" s="0" t="s">
-        <v>615</v>
+        <v>15</v>
       </c>
       <c r="D281" s="0">
-        <v>26350</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="B282" s="0" t="s">
         <v>616</v>
       </c>
-      <c r="B282" s="0" t="s">
+      <c r="C282" s="0" t="s">
         <v>617</v>
       </c>
-      <c r="C282" s="0" t="s">
-        <v>212</v>
-      </c>
       <c r="D282" s="0">
-        <v>31250</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="283">
@@ -7362,10 +7368,10 @@
         <v>619</v>
       </c>
       <c r="C283" s="0" t="s">
-        <v>59</v>
+        <v>212</v>
       </c>
       <c r="D283" s="0">
-        <v>69</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="284">
@@ -7376,10 +7382,10 @@
         <v>621</v>
       </c>
       <c r="C284" s="0" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D284" s="0">
-        <v>34.98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="285">
@@ -7390,7 +7396,7 @@
         <v>623</v>
       </c>
       <c r="C285" s="0" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D285" s="0">
         <v>34.98</v>
@@ -7404,21 +7410,21 @@
         <v>625</v>
       </c>
       <c r="C286" s="0" t="s">
-        <v>626</v>
+        <v>59</v>
       </c>
       <c r="D286" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="0" t="s">
+        <v>626</v>
+      </c>
+      <c r="B287" s="0" t="s">
         <v>627</v>
       </c>
-      <c r="B287" s="0" t="s">
+      <c r="C287" s="0" t="s">
         <v>628</v>
-      </c>
-      <c r="C287" s="0" t="s">
-        <v>52</v>
       </c>
       <c r="D287" s="0">
         <v>65</v>
@@ -7426,30 +7432,30 @@
     </row>
     <row r="288">
       <c r="A288" s="0" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="B288" s="0" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C288" s="0" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D288" s="0">
-        <v>0</v>
+        <v>65</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="0" t="s">
-        <v>630</v>
+        <v>620</v>
       </c>
       <c r="B289" s="0" t="s">
         <v>631</v>
       </c>
       <c r="C289" s="0" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D289" s="0">
-        <v>92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="290">
@@ -7463,7 +7469,7 @@
         <v>52</v>
       </c>
       <c r="D290" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="291">
@@ -7477,7 +7483,7 @@
         <v>52</v>
       </c>
       <c r="D291" s="0">
-        <v>54.8</v>
+        <v>33</v>
       </c>
     </row>
     <row r="292">
@@ -7488,10 +7494,10 @@
         <v>637</v>
       </c>
       <c r="C292" s="0" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D292" s="0">
-        <v>44</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="293">
@@ -7502,10 +7508,10 @@
         <v>639</v>
       </c>
       <c r="C293" s="0" t="s">
-        <v>346</v>
+        <v>59</v>
       </c>
       <c r="D293" s="0">
-        <v>300</v>
+        <v>44</v>
       </c>
     </row>
     <row r="294">
@@ -7519,7 +7525,7 @@
         <v>346</v>
       </c>
       <c r="D294" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="295">
@@ -7530,10 +7536,10 @@
         <v>643</v>
       </c>
       <c r="C295" s="0" t="s">
-        <v>367</v>
+        <v>346</v>
       </c>
       <c r="D295" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="296">
@@ -7544,7 +7550,7 @@
         <v>645</v>
       </c>
       <c r="C296" s="0" t="s">
-        <v>37</v>
+        <v>367</v>
       </c>
       <c r="D296" s="0">
         <v>450</v>
@@ -7558,7 +7564,7 @@
         <v>647</v>
       </c>
       <c r="C297" s="0" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D297" s="0">
         <v>450</v>
@@ -7575,7 +7581,7 @@
         <v>15</v>
       </c>
       <c r="D298" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="299">
@@ -7589,7 +7595,7 @@
         <v>15</v>
       </c>
       <c r="D299" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="300">
@@ -7603,7 +7609,7 @@
         <v>15</v>
       </c>
       <c r="D300" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="301">
@@ -7617,7 +7623,7 @@
         <v>15</v>
       </c>
       <c r="D301" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="302">
@@ -7631,7 +7637,7 @@
         <v>15</v>
       </c>
       <c r="D302" s="0">
-        <v>1300</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="303">
@@ -7645,7 +7651,7 @@
         <v>15</v>
       </c>
       <c r="D303" s="0">
-        <v>2600</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="304">
@@ -7659,7 +7665,7 @@
         <v>15</v>
       </c>
       <c r="D304" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="305">
@@ -7673,7 +7679,7 @@
         <v>15</v>
       </c>
       <c r="D305" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="306">
@@ -7687,7 +7693,7 @@
         <v>15</v>
       </c>
       <c r="D306" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="307">
@@ -7701,7 +7707,7 @@
         <v>15</v>
       </c>
       <c r="D307" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="308">
@@ -7715,7 +7721,7 @@
         <v>15</v>
       </c>
       <c r="D308" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="309">
@@ -7729,7 +7735,7 @@
         <v>15</v>
       </c>
       <c r="D309" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="310">
@@ -7740,10 +7746,10 @@
         <v>673</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="D310" s="0">
-        <v>4730</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="311">
@@ -7757,7 +7763,7 @@
         <v>145</v>
       </c>
       <c r="D311" s="0">
-        <v>2517</v>
+        <v>4730</v>
       </c>
     </row>
     <row r="312">
@@ -7771,7 +7777,7 @@
         <v>145</v>
       </c>
       <c r="D312" s="0">
-        <v>1190</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="313">
@@ -7782,10 +7788,10 @@
         <v>679</v>
       </c>
       <c r="C313" s="0" t="s">
-        <v>28</v>
+        <v>145</v>
       </c>
       <c r="D313" s="0">
-        <v>7655.2</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="314">
@@ -7796,10 +7802,10 @@
         <v>681</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>128</v>
+        <v>28</v>
       </c>
       <c r="D314" s="0">
-        <v>1790</v>
+        <v>7655.2</v>
       </c>
     </row>
     <row r="315">
@@ -7813,7 +7819,7 @@
         <v>128</v>
       </c>
       <c r="D315" s="0">
-        <v>3016.53</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="316">
@@ -7827,7 +7833,7 @@
         <v>128</v>
       </c>
       <c r="D316" s="0">
-        <v>4800</v>
+        <v>3016.53</v>
       </c>
     </row>
     <row r="317">
@@ -7841,7 +7847,7 @@
         <v>128</v>
       </c>
       <c r="D317" s="0">
-        <v>4450</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="318">
@@ -7852,24 +7858,24 @@
         <v>689</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>690</v>
+        <v>128</v>
       </c>
       <c r="D318" s="0">
-        <v>0</v>
+        <v>4450</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="0" t="s">
+        <v>690</v>
+      </c>
+      <c r="B319" s="0" t="s">
         <v>691</v>
       </c>
-      <c r="B319" s="0" t="s">
+      <c r="C319" s="0" t="s">
         <v>692</v>
       </c>
-      <c r="C319" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D319" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="320">
@@ -7883,7 +7889,7 @@
         <v>28</v>
       </c>
       <c r="D320" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="321">
@@ -7894,10 +7900,10 @@
         <v>696</v>
       </c>
       <c r="C321" s="0" t="s">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="D321" s="0">
-        <v>33940.5</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="322">
@@ -7911,7 +7917,7 @@
         <v>97</v>
       </c>
       <c r="D322" s="0">
-        <v>4525.4</v>
+        <v>33940.5</v>
       </c>
     </row>
     <row r="323">
@@ -7922,10 +7928,10 @@
         <v>700</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>156</v>
+        <v>97</v>
       </c>
       <c r="D323" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="324">
@@ -7936,10 +7942,10 @@
         <v>702</v>
       </c>
       <c r="C324" s="0" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="D324" s="0">
-        <v>1125</v>
+        <v>896</v>
       </c>
     </row>
     <row r="325">
@@ -7950,10 +7956,10 @@
         <v>704</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D325" s="0">
-        <v>342732.5</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="326">
@@ -7964,10 +7970,10 @@
         <v>706</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>207</v>
+        <v>97</v>
       </c>
       <c r="D326" s="0">
-        <v>17440</v>
+        <v>342732.5</v>
       </c>
     </row>
     <row r="327">
@@ -7981,7 +7987,7 @@
         <v>207</v>
       </c>
       <c r="D327" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="328">
@@ -8006,10 +8012,10 @@
         <v>712</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>289</v>
+        <v>207</v>
       </c>
       <c r="D329" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="330">
@@ -8020,10 +8026,10 @@
         <v>714</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>207</v>
+        <v>289</v>
       </c>
       <c r="D330" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="331">
@@ -8034,10 +8040,10 @@
         <v>716</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="D331" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="332">
@@ -8048,10 +8054,10 @@
         <v>718</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>97</v>
+        <v>215</v>
       </c>
       <c r="D332" s="0">
-        <v>26620</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="333">
@@ -8065,7 +8071,7 @@
         <v>97</v>
       </c>
       <c r="D333" s="0">
-        <v>266200</v>
+        <v>26620</v>
       </c>
     </row>
     <row r="334">
@@ -8076,10 +8082,10 @@
         <v>722</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="D334" s="0">
-        <v>160</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="335">
@@ -8090,10 +8096,10 @@
         <v>724</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D335" s="0">
-        <v>285.6</v>
+        <v>160</v>
       </c>
     </row>
     <row r="336">
@@ -8107,7 +8113,7 @@
         <v>21</v>
       </c>
       <c r="D336" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="337">
@@ -8118,21 +8124,21 @@
         <v>728</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>729</v>
+        <v>21</v>
       </c>
       <c r="D337" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="0" t="s">
+        <v>729</v>
+      </c>
+      <c r="B338" s="0" t="s">
         <v>730</v>
       </c>
-      <c r="B338" s="0" t="s">
+      <c r="C338" s="0" t="s">
         <v>731</v>
-      </c>
-      <c r="C338" s="0" t="s">
-        <v>732</v>
       </c>
       <c r="D338" s="0">
         <v>770</v>
@@ -8140,16 +8146,16 @@
     </row>
     <row r="339">
       <c r="A339" s="0" t="s">
+        <v>732</v>
+      </c>
+      <c r="B339" s="0" t="s">
         <v>733</v>
       </c>
-      <c r="B339" s="0" t="s">
+      <c r="C339" s="0" t="s">
         <v>734</v>
       </c>
-      <c r="C339" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D339" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="340">
@@ -8160,10 +8166,10 @@
         <v>736</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D340" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="341">
@@ -8174,10 +8180,10 @@
         <v>738</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D341" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="342">
@@ -8188,10 +8194,10 @@
         <v>740</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>156</v>
+        <v>15</v>
       </c>
       <c r="D342" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="343">
@@ -8202,10 +8208,10 @@
         <v>742</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>289</v>
+        <v>156</v>
       </c>
       <c r="D343" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="344">
@@ -8219,7 +8225,7 @@
         <v>289</v>
       </c>
       <c r="D344" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="345">
@@ -8230,10 +8236,10 @@
         <v>746</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>145</v>
+        <v>289</v>
       </c>
       <c r="D345" s="0">
-        <v>935</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="346">
@@ -8247,7 +8253,7 @@
         <v>145</v>
       </c>
       <c r="D346" s="0">
-        <v>620</v>
+        <v>935</v>
       </c>
     </row>
     <row r="347">
@@ -8261,7 +8267,7 @@
         <v>145</v>
       </c>
       <c r="D347" s="0">
-        <v>73</v>
+        <v>620</v>
       </c>
     </row>
     <row r="348">
@@ -8272,10 +8278,10 @@
         <v>752</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D348" s="0">
-        <v>11313.5</v>
+        <v>73</v>
       </c>
     </row>
     <row r="349">
@@ -8286,10 +8292,10 @@
         <v>754</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D349" s="0">
-        <v>400</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="350">
@@ -8300,7 +8306,7 @@
         <v>756</v>
       </c>
       <c r="C350" s="0" t="s">
-        <v>367</v>
+        <v>34</v>
       </c>
       <c r="D350" s="0">
         <v>400</v>
@@ -8314,10 +8320,10 @@
         <v>758</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>21</v>
+        <v>367</v>
       </c>
       <c r="D351" s="0">
-        <v>377</v>
+        <v>400</v>
       </c>
     </row>
     <row r="352">
@@ -8328,10 +8334,10 @@
         <v>760</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D352" s="0">
-        <v>5621.15</v>
+        <v>377</v>
       </c>
     </row>
     <row r="353">
@@ -8342,10 +8348,10 @@
         <v>762</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="D353" s="0">
-        <v>898</v>
+        <v>5621.15</v>
       </c>
     </row>
     <row r="354">
@@ -8356,10 +8362,10 @@
         <v>764</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="D354" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="355">
@@ -8370,10 +8376,10 @@
         <v>766</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>34</v>
+        <v>128</v>
       </c>
       <c r="D355" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="356">
@@ -8384,7 +8390,7 @@
         <v>768</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="D356" s="0">
         <v>650</v>
@@ -8398,10 +8404,10 @@
         <v>770</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="D357" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="358">
@@ -8412,10 +8418,10 @@
         <v>772</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="D358" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="359">
@@ -8426,24 +8432,24 @@
         <v>774</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>775</v>
+        <v>97</v>
       </c>
       <c r="D359" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="0" t="s">
+        <v>775</v>
+      </c>
+      <c r="B360" s="0" t="s">
         <v>776</v>
       </c>
-      <c r="B360" s="0" t="s">
+      <c r="C360" s="0" t="s">
         <v>777</v>
       </c>
-      <c r="C360" s="0" t="s">
-        <v>156</v>
-      </c>
       <c r="D360" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="361">
@@ -8454,10 +8460,10 @@
         <v>779</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="D361" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="362">
@@ -8468,10 +8474,10 @@
         <v>781</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D362" s="0">
-        <v>59000</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="363">
@@ -8482,10 +8488,10 @@
         <v>783</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>156</v>
+        <v>34</v>
       </c>
       <c r="D363" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="364">
@@ -8499,7 +8505,7 @@
         <v>156</v>
       </c>
       <c r="D364" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="365">
@@ -8513,7 +8519,7 @@
         <v>156</v>
       </c>
       <c r="D365" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="366">
@@ -8527,7 +8533,7 @@
         <v>156</v>
       </c>
       <c r="D366" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="367">
@@ -8541,7 +8547,7 @@
         <v>156</v>
       </c>
       <c r="D367" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="368">
@@ -8552,10 +8558,10 @@
         <v>793</v>
       </c>
       <c r="C368" s="0" t="s">
-        <v>269</v>
+        <v>156</v>
       </c>
       <c r="D368" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="369">
@@ -8566,10 +8572,10 @@
         <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>145</v>
+        <v>269</v>
       </c>
       <c r="D369" s="0">
-        <v>365</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="370">
@@ -8580,10 +8586,10 @@
         <v>797</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>289</v>
+        <v>145</v>
       </c>
       <c r="D370" s="0">
-        <v>1450</v>
+        <v>365</v>
       </c>
     </row>
     <row r="371">
@@ -8594,10 +8600,10 @@
         <v>799</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>97</v>
+        <v>289</v>
       </c>
       <c r="D371" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="372">
@@ -8608,10 +8614,10 @@
         <v>801</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>15</v>
+        <v>97</v>
       </c>
       <c r="D372" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="373">
@@ -8622,10 +8628,10 @@
         <v>803</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>289</v>
+        <v>15</v>
       </c>
       <c r="D373" s="0">
-        <v>566</v>
+        <v>900</v>
       </c>
     </row>
     <row r="374">
@@ -8636,10 +8642,10 @@
         <v>805</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>477</v>
+        <v>289</v>
       </c>
       <c r="D374" s="0">
-        <v>64925</v>
+        <v>566</v>
       </c>
     </row>
     <row r="375">
@@ -8650,10 +8656,10 @@
         <v>807</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>15</v>
+        <v>479</v>
       </c>
       <c r="D375" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="376">
@@ -8664,10 +8670,10 @@
         <v>809</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D376" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="377">
@@ -8678,10 +8684,10 @@
         <v>811</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="D377" s="0">
-        <v>1269</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="378">
@@ -8695,7 +8701,7 @@
         <v>145</v>
       </c>
       <c r="D378" s="0">
-        <v>4712</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="379">
@@ -8706,10 +8712,10 @@
         <v>815</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>28</v>
+        <v>145</v>
       </c>
       <c r="D379" s="0">
-        <v>1250</v>
+        <v>4712</v>
       </c>
     </row>
     <row r="380">
@@ -8723,7 +8729,7 @@
         <v>28</v>
       </c>
       <c r="D380" s="0">
-        <v>1986</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="381">
@@ -8734,10 +8740,10 @@
         <v>819</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D381" s="0">
-        <v>450</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="382">
@@ -8751,7 +8757,7 @@
         <v>15</v>
       </c>
       <c r="D382" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="383">
@@ -8776,10 +8782,10 @@
         <v>825</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>387</v>
+        <v>15</v>
       </c>
       <c r="D384" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="385">
@@ -8793,7 +8799,7 @@
         <v>387</v>
       </c>
       <c r="D385" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="386">
@@ -8804,10 +8810,10 @@
         <v>829</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>75</v>
+        <v>387</v>
       </c>
       <c r="D386" s="0">
-        <v>3427</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="387">
@@ -8821,7 +8827,7 @@
         <v>75</v>
       </c>
       <c r="D387" s="0">
-        <v>10618</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="388">
@@ -8832,10 +8838,10 @@
         <v>833</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>289</v>
+        <v>75</v>
       </c>
       <c r="D388" s="0">
-        <v>515</v>
+        <v>10618</v>
       </c>
     </row>
     <row r="389">
@@ -8846,7 +8852,7 @@
         <v>835</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>37</v>
+        <v>289</v>
       </c>
       <c r="D389" s="0">
         <v>515</v>
@@ -8860,10 +8866,10 @@
         <v>837</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D390" s="0">
-        <v>10000</v>
+        <v>515</v>
       </c>
     </row>
     <row r="391">
@@ -8874,10 +8880,10 @@
         <v>839</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>477</v>
+        <v>52</v>
       </c>
       <c r="D391" s="0">
-        <v>213700</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="392">
@@ -8888,10 +8894,10 @@
         <v>841</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D392" s="0">
-        <v>257000</v>
+        <v>213700</v>
       </c>
     </row>
     <row r="393">
@@ -8902,10 +8908,10 @@
         <v>843</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>75</v>
+        <v>479</v>
       </c>
       <c r="D393" s="0">
-        <v>10522</v>
+        <v>257000</v>
       </c>
     </row>
     <row r="394">
@@ -8919,7 +8925,7 @@
         <v>75</v>
       </c>
       <c r="D394" s="0">
-        <v>19481</v>
+        <v>10522</v>
       </c>
     </row>
     <row r="395">
@@ -8930,24 +8936,24 @@
         <v>847</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>848</v>
+        <v>75</v>
       </c>
       <c r="D395" s="0">
-        <v>1080</v>
+        <v>19481</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="0" t="s">
+        <v>848</v>
+      </c>
+      <c r="B396" s="0" t="s">
         <v>849</v>
       </c>
-      <c r="B396" s="0" t="s">
+      <c r="C396" s="0" t="s">
         <v>850</v>
       </c>
-      <c r="C396" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D396" s="0">
-        <v>586.49</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="397">
@@ -8958,24 +8964,24 @@
         <v>852</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>853</v>
+        <v>18</v>
       </c>
       <c r="D397" s="0">
-        <v>520</v>
+        <v>586.49</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="0" t="s">
+        <v>853</v>
+      </c>
+      <c r="B398" s="0" t="s">
         <v>854</v>
       </c>
-      <c r="B398" s="0" t="s">
+      <c r="C398" s="0" t="s">
         <v>855</v>
       </c>
-      <c r="C398" s="0" t="s">
-        <v>853</v>
-      </c>
       <c r="D398" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="399">
@@ -8986,10 +8992,10 @@
         <v>857</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>34</v>
+        <v>855</v>
       </c>
       <c r="D399" s="0">
-        <v>630</v>
+        <v>300</v>
       </c>
     </row>
     <row r="400">
@@ -9000,10 +9006,10 @@
         <v>859</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D400" s="0">
-        <v>2200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="401">
@@ -9017,7 +9023,7 @@
         <v>15</v>
       </c>
       <c r="D401" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="402">
@@ -9028,10 +9034,10 @@
         <v>863</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="D402" s="0">
-        <v>5190.9</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="403">
@@ -9042,10 +9048,10 @@
         <v>865</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="D403" s="0">
-        <v>2969</v>
+        <v>5190.9</v>
       </c>
     </row>
     <row r="404">
@@ -9056,10 +9062,10 @@
         <v>867</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D404" s="0">
-        <v>3800</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="405">
@@ -9070,10 +9076,10 @@
         <v>869</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D405" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="406">
@@ -9084,24 +9090,24 @@
         <v>871</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>872</v>
+        <v>15</v>
       </c>
       <c r="D406" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="0" t="s">
+        <v>872</v>
+      </c>
+      <c r="B407" s="0" t="s">
         <v>873</v>
       </c>
-      <c r="B407" s="0" t="s">
+      <c r="C407" s="0" t="s">
         <v>874</v>
       </c>
-      <c r="C407" s="0" t="s">
-        <v>21</v>
-      </c>
       <c r="D407" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="408">
@@ -9112,10 +9118,10 @@
         <v>876</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>115</v>
+        <v>21</v>
       </c>
       <c r="D408" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="409">
@@ -9126,10 +9132,10 @@
         <v>878</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>15</v>
+        <v>115</v>
       </c>
       <c r="D409" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="410">
@@ -9140,10 +9146,10 @@
         <v>880</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="D410" s="0">
-        <v>146.41</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="411">
@@ -9154,10 +9160,10 @@
         <v>882</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>215</v>
+        <v>97</v>
       </c>
       <c r="D411" s="0">
-        <v>65537</v>
+        <v>146.41</v>
       </c>
     </row>
     <row r="412">
@@ -9168,10 +9174,10 @@
         <v>884</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>145</v>
+        <v>215</v>
       </c>
       <c r="D412" s="0">
-        <v>4130.4</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="413">
@@ -9185,7 +9191,7 @@
         <v>145</v>
       </c>
       <c r="D413" s="0">
-        <v>4283</v>
+        <v>4130.4</v>
       </c>
     </row>
     <row r="414">
@@ -9199,7 +9205,7 @@
         <v>145</v>
       </c>
       <c r="D414" s="0">
-        <v>6524.8</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="415">
@@ -9210,10 +9216,10 @@
         <v>890</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>316</v>
+        <v>145</v>
       </c>
       <c r="D415" s="0">
-        <v>570</v>
+        <v>6524.8</v>
       </c>
     </row>
     <row r="416">
@@ -9224,10 +9230,10 @@
         <v>892</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>75</v>
+        <v>316</v>
       </c>
       <c r="D416" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="417">
@@ -9238,10 +9244,10 @@
         <v>894</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="D417" s="0">
-        <v>153</v>
+        <v>550</v>
       </c>
     </row>
     <row r="418">
@@ -9252,10 +9258,10 @@
         <v>896</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="D418" s="0">
-        <v>740.7</v>
+        <v>153</v>
       </c>
     </row>
     <row r="419">
@@ -9266,10 +9272,10 @@
         <v>898</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="D419" s="0">
-        <v>101000</v>
+        <v>740.7</v>
       </c>
     </row>
     <row r="420">
@@ -9280,10 +9286,10 @@
         <v>900</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="D420" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="421">
@@ -9294,10 +9300,10 @@
         <v>902</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="D421" s="0">
-        <v>883</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="422">
@@ -9308,10 +9314,10 @@
         <v>904</v>
       </c>
       <c r="C422" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D422" s="0">
-        <v>1164.66</v>
+        <v>883</v>
       </c>
     </row>
     <row r="423">
@@ -9322,10 +9328,10 @@
         <v>906</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>156</v>
+        <v>97</v>
       </c>
       <c r="D423" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="424">
@@ -9339,7 +9345,7 @@
         <v>156</v>
       </c>
       <c r="D424" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="425">
@@ -9353,7 +9359,7 @@
         <v>156</v>
       </c>
       <c r="D425" s="0">
-        <v>2150</v>
+        <v>450</v>
       </c>
     </row>
     <row r="426">
@@ -9364,10 +9370,10 @@
         <v>912</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>602</v>
+        <v>156</v>
       </c>
       <c r="D426" s="0">
-        <v>25192.82</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="427">
@@ -9378,10 +9384,10 @@
         <v>914</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>75</v>
+        <v>604</v>
       </c>
       <c r="D427" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="428">
@@ -9392,10 +9398,10 @@
         <v>916</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>180</v>
+        <v>75</v>
       </c>
       <c r="D428" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="429">
@@ -9406,24 +9412,24 @@
         <v>918</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>919</v>
+        <v>180</v>
       </c>
       <c r="D429" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="0" t="s">
+        <v>919</v>
+      </c>
+      <c r="B430" s="0" t="s">
         <v>920</v>
       </c>
-      <c r="B430" s="0" t="s">
+      <c r="C430" s="0" t="s">
         <v>921</v>
       </c>
-      <c r="C430" s="0" t="s">
-        <v>346</v>
-      </c>
       <c r="D430" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="431">
@@ -9434,10 +9440,10 @@
         <v>923</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>40</v>
+        <v>346</v>
       </c>
       <c r="D431" s="0">
-        <v>27991.54</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="432">
@@ -9448,10 +9454,10 @@
         <v>925</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>145</v>
+        <v>40</v>
       </c>
       <c r="D432" s="0">
-        <v>1020</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="433">
@@ -9465,7 +9471,7 @@
         <v>145</v>
       </c>
       <c r="D433" s="0">
-        <v>4106</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="434">
@@ -9476,10 +9482,10 @@
         <v>929</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>289</v>
+        <v>145</v>
       </c>
       <c r="D434" s="0">
-        <v>450</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="435">
@@ -9490,10 +9496,10 @@
         <v>931</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>45</v>
+        <v>289</v>
       </c>
       <c r="D435" s="0">
-        <v>6398.6</v>
+        <v>450</v>
       </c>
     </row>
     <row r="436">
@@ -9507,7 +9513,7 @@
         <v>45</v>
       </c>
       <c r="D436" s="0">
-        <v>2886.7</v>
+        <v>6398.6</v>
       </c>
     </row>
     <row r="437">
@@ -9521,7 +9527,7 @@
         <v>45</v>
       </c>
       <c r="D437" s="0">
-        <v>2050.95</v>
+        <v>2886.7</v>
       </c>
     </row>
     <row r="438">
@@ -9535,7 +9541,7 @@
         <v>45</v>
       </c>
       <c r="D438" s="0">
-        <v>30050.45</v>
+        <v>2050.95</v>
       </c>
     </row>
     <row r="439">
@@ -9549,7 +9555,7 @@
         <v>45</v>
       </c>
       <c r="D439" s="0">
-        <v>2326.8</v>
+        <v>30050.45</v>
       </c>
     </row>
     <row r="440">
@@ -9563,7 +9569,7 @@
         <v>45</v>
       </c>
       <c r="D440" s="0">
-        <v>6429.95</v>
+        <v>2326.8</v>
       </c>
     </row>
     <row r="441">
@@ -9577,7 +9583,7 @@
         <v>45</v>
       </c>
       <c r="D441" s="0">
-        <v>5180.26</v>
+        <v>6429.95</v>
       </c>
     </row>
     <row r="442">
@@ -9588,10 +9594,10 @@
         <v>945</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>212</v>
+        <v>45</v>
       </c>
       <c r="D442" s="0">
-        <v>510</v>
+        <v>5180.26</v>
       </c>
     </row>
     <row r="443">
@@ -9602,7 +9608,7 @@
         <v>947</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>37</v>
+        <v>212</v>
       </c>
       <c r="D443" s="0">
         <v>510</v>
@@ -9616,21 +9622,21 @@
         <v>949</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>950</v>
+        <v>37</v>
       </c>
       <c r="D444" s="0">
-        <v>626</v>
+        <v>510</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="0" t="s">
+        <v>950</v>
+      </c>
+      <c r="B445" s="0" t="s">
         <v>951</v>
       </c>
-      <c r="B445" s="0" t="s">
+      <c r="C445" s="0" t="s">
         <v>952</v>
-      </c>
-      <c r="C445" s="0" t="s">
-        <v>950</v>
       </c>
       <c r="D445" s="0">
         <v>626</v>
@@ -9644,7 +9650,7 @@
         <v>954</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D446" s="0">
         <v>626</v>
@@ -9658,10 +9664,10 @@
         <v>956</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D447" s="0">
-        <v>342</v>
+        <v>626</v>
       </c>
     </row>
     <row r="448">
@@ -9672,7 +9678,7 @@
         <v>958</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D448" s="0">
         <v>342</v>
@@ -9686,7 +9692,7 @@
         <v>960</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D449" s="0">
         <v>342</v>
@@ -9700,10 +9706,10 @@
         <v>962</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D450" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="451">
@@ -9714,7 +9720,7 @@
         <v>964</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D451" s="0">
         <v>0</v>
@@ -9728,21 +9734,21 @@
         <v>966</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>967</v>
+        <v>952</v>
       </c>
       <c r="D452" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="0" t="s">
+        <v>967</v>
+      </c>
+      <c r="B453" s="0" t="s">
         <v>968</v>
       </c>
-      <c r="B453" s="0" t="s">
+      <c r="C453" s="0" t="s">
         <v>969</v>
-      </c>
-      <c r="C453" s="0" t="s">
-        <v>950</v>
       </c>
       <c r="D453" s="0">
         <v>453</v>
@@ -9756,10 +9762,10 @@
         <v>971</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>75</v>
+        <v>952</v>
       </c>
       <c r="D454" s="0">
-        <v>19322</v>
+        <v>453</v>
       </c>
     </row>
     <row r="455">
@@ -9770,10 +9776,10 @@
         <v>973</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D455" s="0">
-        <v>430</v>
+        <v>19322</v>
       </c>
     </row>
     <row r="456">
@@ -9784,7 +9790,7 @@
         <v>975</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>289</v>
+        <v>34</v>
       </c>
       <c r="D456" s="0">
         <v>430</v>
@@ -9798,10 +9804,10 @@
         <v>977</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>120</v>
+        <v>289</v>
       </c>
       <c r="D457" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="458">
@@ -9812,10 +9818,10 @@
         <v>979</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="D458" s="0">
-        <v>12049</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="459">
@@ -9829,7 +9835,7 @@
         <v>145</v>
       </c>
       <c r="D459" s="0">
-        <v>2895</v>
+        <v>12049</v>
       </c>
     </row>
     <row r="460">
@@ -9840,10 +9846,10 @@
         <v>983</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D460" s="0">
-        <v>266200</v>
+        <v>2895</v>
       </c>
     </row>
     <row r="461">
@@ -9857,7 +9863,7 @@
         <v>97</v>
       </c>
       <c r="D461" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="462">
@@ -9871,7 +9877,7 @@
         <v>97</v>
       </c>
       <c r="D462" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="463">
@@ -9882,24 +9888,24 @@
         <v>989</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>990</v>
+        <v>97</v>
       </c>
       <c r="D463" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="0" t="s">
+        <v>990</v>
+      </c>
+      <c r="B464" s="0" t="s">
         <v>991</v>
       </c>
-      <c r="B464" s="0" t="s">
+      <c r="C464" s="0" t="s">
         <v>992</v>
       </c>
-      <c r="C464" s="0" t="s">
-        <v>990</v>
-      </c>
       <c r="D464" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="465">
@@ -9910,10 +9916,10 @@
         <v>994</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="D465" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="466">
@@ -9924,10 +9930,10 @@
         <v>996</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="D466" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="467">
@@ -9938,10 +9944,10 @@
         <v>998</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="D467" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="468">
@@ -9952,10 +9958,10 @@
         <v>1000</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>75</v>
+        <v>992</v>
       </c>
       <c r="D468" s="0">
-        <v>4276</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="469">
@@ -9966,10 +9972,10 @@
         <v>1002</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>145</v>
+        <v>75</v>
       </c>
       <c r="D469" s="0">
-        <v>3930</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="470">
@@ -9980,10 +9986,10 @@
         <v>1004</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D470" s="0">
-        <v>4392.3</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="471">
@@ -9994,24 +10000,24 @@
         <v>1006</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>1007</v>
+        <v>97</v>
       </c>
       <c r="D471" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="0" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B472" s="0" t="s">
         <v>1008</v>
       </c>
-      <c r="B472" s="0" t="s">
+      <c r="C472" s="0" t="s">
         <v>1009</v>
       </c>
-      <c r="C472" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D472" s="0">
-        <v>1297</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="473">
@@ -10025,7 +10031,7 @@
         <v>52</v>
       </c>
       <c r="D473" s="0">
-        <v>298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="474">
@@ -10039,7 +10045,7 @@
         <v>52</v>
       </c>
       <c r="D474" s="0">
-        <v>596</v>
+        <v>298</v>
       </c>
     </row>
     <row r="475">
@@ -10050,10 +10056,10 @@
         <v>1015</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>384</v>
+        <v>52</v>
       </c>
       <c r="D475" s="0">
-        <v>65142.6</v>
+        <v>596</v>
       </c>
     </row>
     <row r="476">
@@ -10067,7 +10073,7 @@
         <v>384</v>
       </c>
       <c r="D476" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="477">
@@ -10078,10 +10084,10 @@
         <v>1019</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>28</v>
+        <v>384</v>
       </c>
       <c r="D477" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="478">
@@ -10092,10 +10098,10 @@
         <v>1021</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D478" s="0">
-        <v>12000</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="479">
@@ -10109,7 +10115,7 @@
         <v>52</v>
       </c>
       <c r="D479" s="0">
-        <v>17425</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="480">
@@ -10120,66 +10126,66 @@
         <v>1025</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>1026</v>
+        <v>52</v>
       </c>
       <c r="D480" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="0" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B481" s="0" t="s">
         <v>1027</v>
       </c>
-      <c r="B481" s="0" t="s">
+      <c r="C481" s="0" t="s">
         <v>1028</v>
       </c>
-      <c r="C481" s="0" t="s">
-        <v>1029</v>
-      </c>
       <c r="D481" s="0">
-        <v>2282.3</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="0" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B482" s="0" t="s">
         <v>1030</v>
       </c>
-      <c r="B482" s="0" t="s">
+      <c r="C482" s="0" t="s">
         <v>1031</v>
       </c>
-      <c r="C482" s="0" t="s">
-        <v>1032</v>
-      </c>
       <c r="D482" s="0">
-        <v>386</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="0" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B483" s="0" t="s">
         <v>1033</v>
       </c>
-      <c r="B483" s="0" t="s">
+      <c r="C483" s="0" t="s">
         <v>1034</v>
       </c>
-      <c r="C483" s="0" t="s">
-        <v>1035</v>
-      </c>
       <c r="D483" s="0">
-        <v>385.4</v>
+        <v>386</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B484" s="0" t="s">
         <v>1036</v>
       </c>
-      <c r="B484" s="0" t="s">
+      <c r="C484" s="0" t="s">
         <v>1037</v>
       </c>
-      <c r="C484" s="0" t="s">
-        <v>97</v>
-      </c>
       <c r="D484" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="485">
@@ -10190,10 +10196,10 @@
         <v>1039</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="D485" s="0">
-        <v>1890</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="486">
@@ -10204,10 +10210,10 @@
         <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>602</v>
+        <v>128</v>
       </c>
       <c r="D486" s="0">
-        <v>83000</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="487">
@@ -10218,10 +10224,10 @@
         <v>1043</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>145</v>
+        <v>604</v>
       </c>
       <c r="D487" s="0">
-        <v>99</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="488">
@@ -10232,10 +10238,10 @@
         <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="D488" s="0">
-        <v>950</v>
+        <v>99</v>
       </c>
     </row>
     <row r="489">
@@ -10246,10 +10252,10 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>477</v>
+        <v>75</v>
       </c>
       <c r="D489" s="0">
-        <v>398107</v>
+        <v>950</v>
       </c>
     </row>
     <row r="490">
@@ -10260,10 +10266,10 @@
         <v>1049</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>165</v>
+        <v>479</v>
       </c>
       <c r="D490" s="0">
-        <v>2200</v>
+        <v>398107</v>
       </c>
     </row>
     <row r="491">
@@ -10274,10 +10280,10 @@
         <v>1051</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>212</v>
+        <v>165</v>
       </c>
       <c r="D491" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="492">
@@ -10288,10 +10294,10 @@
         <v>1053</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>75</v>
+        <v>212</v>
       </c>
       <c r="D492" s="0">
-        <v>5790</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="493">
@@ -10302,10 +10308,10 @@
         <v>1055</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>950</v>
+        <v>75</v>
       </c>
       <c r="D493" s="0">
-        <v>880</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="494">
@@ -10316,7 +10322,7 @@
         <v>1057</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D494" s="0">
         <v>880</v>
@@ -10330,7 +10336,7 @@
         <v>1059</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D495" s="0">
         <v>880</v>
@@ -10344,10 +10350,10 @@
         <v>1061</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>21</v>
+        <v>952</v>
       </c>
       <c r="D496" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="497">
@@ -10358,10 +10364,10 @@
         <v>1063</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D497" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="498">
@@ -10375,7 +10381,7 @@
         <v>15</v>
       </c>
       <c r="D498" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="499">
@@ -10386,10 +10392,10 @@
         <v>1067</v>
       </c>
       <c r="C499" s="0" t="s">
-        <v>289</v>
+        <v>15</v>
       </c>
       <c r="D499" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="500">
@@ -10403,7 +10409,7 @@
         <v>289</v>
       </c>
       <c r="D500" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="501">
@@ -10414,10 +10420,10 @@
         <v>1071</v>
       </c>
       <c r="C501" s="0" t="s">
-        <v>15</v>
+        <v>289</v>
       </c>
       <c r="D501" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="502">
@@ -10431,7 +10437,7 @@
         <v>15</v>
       </c>
       <c r="D502" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="503">
@@ -10442,24 +10448,24 @@
         <v>1075</v>
       </c>
       <c r="C503" s="0" t="s">
-        <v>1076</v>
+        <v>15</v>
       </c>
       <c r="D503" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="0" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B504" s="0" t="s">
         <v>1077</v>
       </c>
-      <c r="B504" s="0" t="s">
+      <c r="C504" s="0" t="s">
         <v>1078</v>
       </c>
-      <c r="C504" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D504" s="0">
-        <v>15189</v>
+        <v>1</v>
       </c>
     </row>
     <row r="505">
@@ -10470,10 +10476,10 @@
         <v>1080</v>
       </c>
       <c r="C505" s="0" t="s">
-        <v>384</v>
+        <v>28</v>
       </c>
       <c r="D505" s="0">
-        <v>3859.93</v>
+        <v>15189</v>
       </c>
     </row>
     <row r="506">
@@ -10487,7 +10493,7 @@
         <v>384</v>
       </c>
       <c r="D506" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="507">
@@ -10498,10 +10504,10 @@
         <v>1084</v>
       </c>
       <c r="C507" s="0" t="s">
-        <v>346</v>
+        <v>384</v>
       </c>
       <c r="D507" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="508">
@@ -10515,7 +10521,7 @@
         <v>346</v>
       </c>
       <c r="D508" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="509">
@@ -10526,10 +10532,10 @@
         <v>1088</v>
       </c>
       <c r="C509" s="0" t="s">
-        <v>37</v>
+        <v>346</v>
       </c>
       <c r="D509" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="510">
@@ -10540,24 +10546,24 @@
         <v>1090</v>
       </c>
       <c r="C510" s="0" t="s">
-        <v>1091</v>
+        <v>37</v>
       </c>
       <c r="D510" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="0" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B511" s="0" t="s">
         <v>1092</v>
       </c>
-      <c r="B511" s="0" t="s">
+      <c r="C511" s="0" t="s">
         <v>1093</v>
       </c>
-      <c r="C511" s="0" t="s">
-        <v>110</v>
-      </c>
       <c r="D511" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="512">
@@ -10568,10 +10574,10 @@
         <v>1095</v>
       </c>
       <c r="C512" s="0" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="D512" s="0">
-        <v>43590.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="513">
@@ -10582,10 +10588,10 @@
         <v>1097</v>
       </c>
       <c r="C513" s="0" t="s">
-        <v>477</v>
+        <v>97</v>
       </c>
       <c r="D513" s="0">
-        <v>213700</v>
+        <v>43590.25</v>
       </c>
     </row>
     <row r="514">
@@ -10596,10 +10602,10 @@
         <v>1099</v>
       </c>
       <c r="C514" s="0" t="s">
-        <v>384</v>
+        <v>479</v>
       </c>
       <c r="D514" s="0">
-        <v>77429.29</v>
+        <v>213700</v>
       </c>
     </row>
     <row r="515">
@@ -10613,7 +10619,7 @@
         <v>384</v>
       </c>
       <c r="D515" s="0">
-        <v>42913.42</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="516">
@@ -10627,7 +10633,7 @@
         <v>384</v>
       </c>
       <c r="D516" s="0">
-        <v>88806.25</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="517">
@@ -10641,7 +10647,7 @@
         <v>384</v>
       </c>
       <c r="D517" s="0">
-        <v>50781.52</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="518">
@@ -10652,10 +10658,10 @@
         <v>1107</v>
       </c>
       <c r="C518" s="0" t="s">
-        <v>21</v>
+        <v>384</v>
       </c>
       <c r="D518" s="0">
-        <v>1600</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="519">
@@ -10666,10 +10672,10 @@
         <v>1109</v>
       </c>
       <c r="C519" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D519" s="0">
-        <v>3521.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="520">
@@ -10683,7 +10689,7 @@
         <v>28</v>
       </c>
       <c r="D520" s="0">
-        <v>3987</v>
+        <v>3521.4</v>
       </c>
     </row>
     <row r="521">
@@ -10697,7 +10703,7 @@
         <v>28</v>
       </c>
       <c r="D521" s="0">
-        <v>4086.37</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="522">
@@ -10711,7 +10717,7 @@
         <v>28</v>
       </c>
       <c r="D522" s="0">
-        <v>3382.65</v>
+        <v>4086.37</v>
       </c>
     </row>
     <row r="523">
@@ -10722,10 +10728,10 @@
         <v>1117</v>
       </c>
       <c r="C523" s="0" t="s">
-        <v>165</v>
+        <v>28</v>
       </c>
       <c r="D523" s="0">
-        <v>430</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="524">
@@ -10736,9 +10742,23 @@
         <v>1119</v>
       </c>
       <c r="C524" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D524" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="0" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B525" s="0" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C525" s="0" t="s">
         <v>145</v>
       </c>
-      <c r="D524" s="0">
+      <c r="D525" s="0">
         <v>495</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados mié 21/10/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3815,7 +3815,7 @@
         <v>69</v>
       </c>
       <c r="D29" s="0">
-        <v>2158.2</v>
+        <v>2275</v>
       </c>
     </row>
     <row r="30">
@@ -3829,7 +3829,7 @@
         <v>72</v>
       </c>
       <c r="D30" s="0">
-        <v>2220</v>
+        <v>2275</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
sync: stock y precios actualizados vie 23/10/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="1122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="1124">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -2307,6 +2307,12 @@
   </si>
   <si>
     <t xml:space="preserve">METRONIDAZOL DENVER FARMA 500MG COMP. X   10 - 000022239</t>
+  </si>
+  <si>
+    <t>000024247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">METRONIDAZOL VANNIER 500MG  X 10 COMPRIMIDOS - 000024247</t>
   </si>
   <si>
     <t>000022207</t>
@@ -3443,7 +3449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D525"/>
+  <dimension ref="A2:D526"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -6895,7 +6901,7 @@
         <v>75</v>
       </c>
       <c r="D249" s="0">
-        <v>90000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="250">
@@ -6909,7 +6915,7 @@
         <v>75</v>
       </c>
       <c r="D250" s="0">
-        <v>110000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="251">
@@ -8376,10 +8382,10 @@
         <v>766</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>128</v>
+        <v>21</v>
       </c>
       <c r="D355" s="0">
-        <v>4767</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="356">
@@ -8390,10 +8396,10 @@
         <v>768</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>34</v>
+        <v>128</v>
       </c>
       <c r="D356" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="357">
@@ -8404,7 +8410,7 @@
         <v>770</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="D357" s="0">
         <v>650</v>
@@ -8418,10 +8424,10 @@
         <v>772</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="D358" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="359">
@@ -8432,10 +8438,10 @@
         <v>774</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="D359" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="360">
@@ -8446,24 +8452,24 @@
         <v>776</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>777</v>
+        <v>97</v>
       </c>
       <c r="D360" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="0" t="s">
+        <v>777</v>
+      </c>
+      <c r="B361" s="0" t="s">
         <v>778</v>
       </c>
-      <c r="B361" s="0" t="s">
+      <c r="C361" s="0" t="s">
         <v>779</v>
       </c>
-      <c r="C361" s="0" t="s">
-        <v>156</v>
-      </c>
       <c r="D361" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="362">
@@ -8474,10 +8480,10 @@
         <v>781</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="D362" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="363">
@@ -8488,10 +8494,10 @@
         <v>783</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D363" s="0">
-        <v>59000</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="364">
@@ -8502,10 +8508,10 @@
         <v>785</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>156</v>
+        <v>34</v>
       </c>
       <c r="D364" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="365">
@@ -8519,7 +8525,7 @@
         <v>156</v>
       </c>
       <c r="D365" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="366">
@@ -8533,7 +8539,7 @@
         <v>156</v>
       </c>
       <c r="D366" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="367">
@@ -8547,7 +8553,7 @@
         <v>156</v>
       </c>
       <c r="D367" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="368">
@@ -8561,7 +8567,7 @@
         <v>156</v>
       </c>
       <c r="D368" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="369">
@@ -8572,10 +8578,10 @@
         <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>269</v>
+        <v>156</v>
       </c>
       <c r="D369" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="370">
@@ -8586,10 +8592,10 @@
         <v>797</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>145</v>
+        <v>269</v>
       </c>
       <c r="D370" s="0">
-        <v>365</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="371">
@@ -8600,10 +8606,10 @@
         <v>799</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>289</v>
+        <v>145</v>
       </c>
       <c r="D371" s="0">
-        <v>1450</v>
+        <v>365</v>
       </c>
     </row>
     <row r="372">
@@ -8614,10 +8620,10 @@
         <v>801</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>97</v>
+        <v>289</v>
       </c>
       <c r="D372" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="373">
@@ -8628,10 +8634,10 @@
         <v>803</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>15</v>
+        <v>97</v>
       </c>
       <c r="D373" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="374">
@@ -8642,10 +8648,10 @@
         <v>805</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>289</v>
+        <v>15</v>
       </c>
       <c r="D374" s="0">
-        <v>566</v>
+        <v>900</v>
       </c>
     </row>
     <row r="375">
@@ -8656,10 +8662,10 @@
         <v>807</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>479</v>
+        <v>289</v>
       </c>
       <c r="D375" s="0">
-        <v>64925</v>
+        <v>566</v>
       </c>
     </row>
     <row r="376">
@@ -8670,10 +8676,10 @@
         <v>809</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>15</v>
+        <v>479</v>
       </c>
       <c r="D376" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="377">
@@ -8684,10 +8690,10 @@
         <v>811</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D377" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="378">
@@ -8698,10 +8704,10 @@
         <v>813</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="D378" s="0">
-        <v>1269</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="379">
@@ -8715,7 +8721,7 @@
         <v>145</v>
       </c>
       <c r="D379" s="0">
-        <v>4712</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="380">
@@ -8726,10 +8732,10 @@
         <v>817</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>28</v>
+        <v>145</v>
       </c>
       <c r="D380" s="0">
-        <v>1250</v>
+        <v>4712</v>
       </c>
     </row>
     <row r="381">
@@ -8743,7 +8749,7 @@
         <v>28</v>
       </c>
       <c r="D381" s="0">
-        <v>1986</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="382">
@@ -8754,10 +8760,10 @@
         <v>821</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D382" s="0">
-        <v>450</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="383">
@@ -8771,7 +8777,7 @@
         <v>15</v>
       </c>
       <c r="D383" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="384">
@@ -8796,10 +8802,10 @@
         <v>827</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>387</v>
+        <v>15</v>
       </c>
       <c r="D385" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="386">
@@ -8813,7 +8819,7 @@
         <v>387</v>
       </c>
       <c r="D386" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="387">
@@ -8824,10 +8830,10 @@
         <v>831</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>75</v>
+        <v>387</v>
       </c>
       <c r="D387" s="0">
-        <v>3427</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="388">
@@ -8841,7 +8847,7 @@
         <v>75</v>
       </c>
       <c r="D388" s="0">
-        <v>10618</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="389">
@@ -8852,10 +8858,10 @@
         <v>835</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>289</v>
+        <v>75</v>
       </c>
       <c r="D389" s="0">
-        <v>515</v>
+        <v>10618</v>
       </c>
     </row>
     <row r="390">
@@ -8866,7 +8872,7 @@
         <v>837</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>37</v>
+        <v>289</v>
       </c>
       <c r="D390" s="0">
         <v>515</v>
@@ -8880,10 +8886,10 @@
         <v>839</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D391" s="0">
-        <v>10000</v>
+        <v>515</v>
       </c>
     </row>
     <row r="392">
@@ -8894,10 +8900,10 @@
         <v>841</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>479</v>
+        <v>52</v>
       </c>
       <c r="D392" s="0">
-        <v>213700</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="393">
@@ -8911,7 +8917,7 @@
         <v>479</v>
       </c>
       <c r="D393" s="0">
-        <v>257000</v>
+        <v>213700</v>
       </c>
     </row>
     <row r="394">
@@ -8922,10 +8928,10 @@
         <v>845</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>75</v>
+        <v>479</v>
       </c>
       <c r="D394" s="0">
-        <v>10522</v>
+        <v>257000</v>
       </c>
     </row>
     <row r="395">
@@ -8939,7 +8945,7 @@
         <v>75</v>
       </c>
       <c r="D395" s="0">
-        <v>19481</v>
+        <v>10522</v>
       </c>
     </row>
     <row r="396">
@@ -8950,24 +8956,24 @@
         <v>849</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>850</v>
+        <v>75</v>
       </c>
       <c r="D396" s="0">
-        <v>1080</v>
+        <v>19481</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="0" t="s">
+        <v>850</v>
+      </c>
+      <c r="B397" s="0" t="s">
         <v>851</v>
       </c>
-      <c r="B397" s="0" t="s">
+      <c r="C397" s="0" t="s">
         <v>852</v>
       </c>
-      <c r="C397" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D397" s="0">
-        <v>586.49</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="398">
@@ -8978,24 +8984,24 @@
         <v>854</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>855</v>
+        <v>18</v>
       </c>
       <c r="D398" s="0">
-        <v>520</v>
+        <v>586.49</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="0" t="s">
+        <v>855</v>
+      </c>
+      <c r="B399" s="0" t="s">
         <v>856</v>
       </c>
-      <c r="B399" s="0" t="s">
+      <c r="C399" s="0" t="s">
         <v>857</v>
       </c>
-      <c r="C399" s="0" t="s">
-        <v>855</v>
-      </c>
       <c r="D399" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="400">
@@ -9006,10 +9012,10 @@
         <v>859</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>34</v>
+        <v>857</v>
       </c>
       <c r="D400" s="0">
-        <v>630</v>
+        <v>300</v>
       </c>
     </row>
     <row r="401">
@@ -9020,10 +9026,10 @@
         <v>861</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D401" s="0">
-        <v>2200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="402">
@@ -9037,7 +9043,7 @@
         <v>15</v>
       </c>
       <c r="D402" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="403">
@@ -9048,10 +9054,10 @@
         <v>865</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="D403" s="0">
-        <v>5190.9</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="404">
@@ -9062,10 +9068,10 @@
         <v>867</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="D404" s="0">
-        <v>2969</v>
+        <v>5190.9</v>
       </c>
     </row>
     <row r="405">
@@ -9076,10 +9082,10 @@
         <v>869</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D405" s="0">
-        <v>3800</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="406">
@@ -9090,10 +9096,10 @@
         <v>871</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D406" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="407">
@@ -9104,24 +9110,24 @@
         <v>873</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>874</v>
+        <v>15</v>
       </c>
       <c r="D407" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="0" t="s">
+        <v>874</v>
+      </c>
+      <c r="B408" s="0" t="s">
         <v>875</v>
       </c>
-      <c r="B408" s="0" t="s">
+      <c r="C408" s="0" t="s">
         <v>876</v>
       </c>
-      <c r="C408" s="0" t="s">
-        <v>21</v>
-      </c>
       <c r="D408" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="409">
@@ -9132,10 +9138,10 @@
         <v>878</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>115</v>
+        <v>21</v>
       </c>
       <c r="D409" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="410">
@@ -9146,10 +9152,10 @@
         <v>880</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>15</v>
+        <v>115</v>
       </c>
       <c r="D410" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="411">
@@ -9160,10 +9166,10 @@
         <v>882</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="D411" s="0">
-        <v>146.41</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="412">
@@ -9174,10 +9180,10 @@
         <v>884</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>215</v>
+        <v>97</v>
       </c>
       <c r="D412" s="0">
-        <v>65537</v>
+        <v>146.41</v>
       </c>
     </row>
     <row r="413">
@@ -9188,10 +9194,10 @@
         <v>886</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>145</v>
+        <v>215</v>
       </c>
       <c r="D413" s="0">
-        <v>4130.4</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="414">
@@ -9205,7 +9211,7 @@
         <v>145</v>
       </c>
       <c r="D414" s="0">
-        <v>4283</v>
+        <v>4130.4</v>
       </c>
     </row>
     <row r="415">
@@ -9219,7 +9225,7 @@
         <v>145</v>
       </c>
       <c r="D415" s="0">
-        <v>6524.8</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="416">
@@ -9230,10 +9236,10 @@
         <v>892</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>316</v>
+        <v>145</v>
       </c>
       <c r="D416" s="0">
-        <v>570</v>
+        <v>6524.8</v>
       </c>
     </row>
     <row r="417">
@@ -9244,10 +9250,10 @@
         <v>894</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>75</v>
+        <v>316</v>
       </c>
       <c r="D417" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="418">
@@ -9258,10 +9264,10 @@
         <v>896</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="D418" s="0">
-        <v>153</v>
+        <v>550</v>
       </c>
     </row>
     <row r="419">
@@ -9272,10 +9278,10 @@
         <v>898</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="D419" s="0">
-        <v>740.7</v>
+        <v>153</v>
       </c>
     </row>
     <row r="420">
@@ -9286,10 +9292,10 @@
         <v>900</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="D420" s="0">
-        <v>101000</v>
+        <v>740.7</v>
       </c>
     </row>
     <row r="421">
@@ -9300,10 +9306,10 @@
         <v>902</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="D421" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="422">
@@ -9314,10 +9320,10 @@
         <v>904</v>
       </c>
       <c r="C422" s="0" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="D422" s="0">
-        <v>883</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="423">
@@ -9328,10 +9334,10 @@
         <v>906</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D423" s="0">
-        <v>1164.66</v>
+        <v>883</v>
       </c>
     </row>
     <row r="424">
@@ -9342,10 +9348,10 @@
         <v>908</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>156</v>
+        <v>97</v>
       </c>
       <c r="D424" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="425">
@@ -9359,7 +9365,7 @@
         <v>156</v>
       </c>
       <c r="D425" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="426">
@@ -9373,7 +9379,7 @@
         <v>156</v>
       </c>
       <c r="D426" s="0">
-        <v>2150</v>
+        <v>450</v>
       </c>
     </row>
     <row r="427">
@@ -9384,10 +9390,10 @@
         <v>914</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>604</v>
+        <v>156</v>
       </c>
       <c r="D427" s="0">
-        <v>25192.82</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="428">
@@ -9398,10 +9404,10 @@
         <v>916</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>75</v>
+        <v>604</v>
       </c>
       <c r="D428" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="429">
@@ -9412,10 +9418,10 @@
         <v>918</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>180</v>
+        <v>75</v>
       </c>
       <c r="D429" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="430">
@@ -9426,24 +9432,24 @@
         <v>920</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>921</v>
+        <v>180</v>
       </c>
       <c r="D430" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="0" t="s">
+        <v>921</v>
+      </c>
+      <c r="B431" s="0" t="s">
         <v>922</v>
       </c>
-      <c r="B431" s="0" t="s">
+      <c r="C431" s="0" t="s">
         <v>923</v>
       </c>
-      <c r="C431" s="0" t="s">
-        <v>346</v>
-      </c>
       <c r="D431" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="432">
@@ -9454,10 +9460,10 @@
         <v>925</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>40</v>
+        <v>346</v>
       </c>
       <c r="D432" s="0">
-        <v>27991.54</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="433">
@@ -9468,10 +9474,10 @@
         <v>927</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>145</v>
+        <v>40</v>
       </c>
       <c r="D433" s="0">
-        <v>1020</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="434">
@@ -9485,7 +9491,7 @@
         <v>145</v>
       </c>
       <c r="D434" s="0">
-        <v>4106</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="435">
@@ -9496,10 +9502,10 @@
         <v>931</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>289</v>
+        <v>145</v>
       </c>
       <c r="D435" s="0">
-        <v>450</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="436">
@@ -9510,10 +9516,10 @@
         <v>933</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>45</v>
+        <v>289</v>
       </c>
       <c r="D436" s="0">
-        <v>6398.6</v>
+        <v>450</v>
       </c>
     </row>
     <row r="437">
@@ -9527,7 +9533,7 @@
         <v>45</v>
       </c>
       <c r="D437" s="0">
-        <v>2886.7</v>
+        <v>6398.6</v>
       </c>
     </row>
     <row r="438">
@@ -9541,7 +9547,7 @@
         <v>45</v>
       </c>
       <c r="D438" s="0">
-        <v>2050.95</v>
+        <v>2886.7</v>
       </c>
     </row>
     <row r="439">
@@ -9555,7 +9561,7 @@
         <v>45</v>
       </c>
       <c r="D439" s="0">
-        <v>30050.45</v>
+        <v>2050.95</v>
       </c>
     </row>
     <row r="440">
@@ -9569,7 +9575,7 @@
         <v>45</v>
       </c>
       <c r="D440" s="0">
-        <v>2326.8</v>
+        <v>30050.45</v>
       </c>
     </row>
     <row r="441">
@@ -9583,7 +9589,7 @@
         <v>45</v>
       </c>
       <c r="D441" s="0">
-        <v>6429.95</v>
+        <v>2326.8</v>
       </c>
     </row>
     <row r="442">
@@ -9597,7 +9603,7 @@
         <v>45</v>
       </c>
       <c r="D442" s="0">
-        <v>5180.26</v>
+        <v>6429.95</v>
       </c>
     </row>
     <row r="443">
@@ -9608,10 +9614,10 @@
         <v>947</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>212</v>
+        <v>45</v>
       </c>
       <c r="D443" s="0">
-        <v>510</v>
+        <v>5180.26</v>
       </c>
     </row>
     <row r="444">
@@ -9622,7 +9628,7 @@
         <v>949</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>37</v>
+        <v>212</v>
       </c>
       <c r="D444" s="0">
         <v>510</v>
@@ -9636,21 +9642,21 @@
         <v>951</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>952</v>
+        <v>37</v>
       </c>
       <c r="D445" s="0">
-        <v>626</v>
+        <v>510</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="0" t="s">
+        <v>952</v>
+      </c>
+      <c r="B446" s="0" t="s">
         <v>953</v>
       </c>
-      <c r="B446" s="0" t="s">
+      <c r="C446" s="0" t="s">
         <v>954</v>
-      </c>
-      <c r="C446" s="0" t="s">
-        <v>952</v>
       </c>
       <c r="D446" s="0">
         <v>626</v>
@@ -9664,7 +9670,7 @@
         <v>956</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D447" s="0">
         <v>626</v>
@@ -9678,10 +9684,10 @@
         <v>958</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D448" s="0">
-        <v>342</v>
+        <v>626</v>
       </c>
     </row>
     <row r="449">
@@ -9692,7 +9698,7 @@
         <v>960</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D449" s="0">
         <v>342</v>
@@ -9706,7 +9712,7 @@
         <v>962</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D450" s="0">
         <v>342</v>
@@ -9720,10 +9726,10 @@
         <v>964</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D451" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="452">
@@ -9734,7 +9740,7 @@
         <v>966</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D452" s="0">
         <v>0</v>
@@ -9748,21 +9754,21 @@
         <v>968</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>969</v>
+        <v>954</v>
       </c>
       <c r="D453" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="0" t="s">
+        <v>969</v>
+      </c>
+      <c r="B454" s="0" t="s">
         <v>970</v>
       </c>
-      <c r="B454" s="0" t="s">
+      <c r="C454" s="0" t="s">
         <v>971</v>
-      </c>
-      <c r="C454" s="0" t="s">
-        <v>952</v>
       </c>
       <c r="D454" s="0">
         <v>453</v>
@@ -9776,10 +9782,10 @@
         <v>973</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>75</v>
+        <v>954</v>
       </c>
       <c r="D455" s="0">
-        <v>19322</v>
+        <v>453</v>
       </c>
     </row>
     <row r="456">
@@ -9790,10 +9796,10 @@
         <v>975</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D456" s="0">
-        <v>430</v>
+        <v>19322</v>
       </c>
     </row>
     <row r="457">
@@ -9804,7 +9810,7 @@
         <v>977</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>289</v>
+        <v>34</v>
       </c>
       <c r="D457" s="0">
         <v>430</v>
@@ -9818,10 +9824,10 @@
         <v>979</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>120</v>
+        <v>289</v>
       </c>
       <c r="D458" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="459">
@@ -9832,10 +9838,10 @@
         <v>981</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="D459" s="0">
-        <v>12049</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="460">
@@ -9849,7 +9855,7 @@
         <v>145</v>
       </c>
       <c r="D460" s="0">
-        <v>2895</v>
+        <v>12049</v>
       </c>
     </row>
     <row r="461">
@@ -9860,10 +9866,10 @@
         <v>985</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D461" s="0">
-        <v>266200</v>
+        <v>2895</v>
       </c>
     </row>
     <row r="462">
@@ -9877,7 +9883,7 @@
         <v>97</v>
       </c>
       <c r="D462" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="463">
@@ -9891,7 +9897,7 @@
         <v>97</v>
       </c>
       <c r="D463" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="464">
@@ -9902,24 +9908,24 @@
         <v>991</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>992</v>
+        <v>97</v>
       </c>
       <c r="D464" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
+        <v>992</v>
+      </c>
+      <c r="B465" s="0" t="s">
         <v>993</v>
       </c>
-      <c r="B465" s="0" t="s">
+      <c r="C465" s="0" t="s">
         <v>994</v>
       </c>
-      <c r="C465" s="0" t="s">
-        <v>992</v>
-      </c>
       <c r="D465" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="466">
@@ -9930,10 +9936,10 @@
         <v>996</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="D466" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="467">
@@ -9944,10 +9950,10 @@
         <v>998</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="D467" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="468">
@@ -9958,10 +9964,10 @@
         <v>1000</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="D468" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="469">
@@ -9972,10 +9978,10 @@
         <v>1002</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>75</v>
+        <v>994</v>
       </c>
       <c r="D469" s="0">
-        <v>4276</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="470">
@@ -9986,10 +9992,10 @@
         <v>1004</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>145</v>
+        <v>75</v>
       </c>
       <c r="D470" s="0">
-        <v>3930</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="471">
@@ -10000,10 +10006,10 @@
         <v>1006</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="D471" s="0">
-        <v>4392.3</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="472">
@@ -10014,24 +10020,24 @@
         <v>1008</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>1009</v>
+        <v>97</v>
       </c>
       <c r="D472" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="0" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B473" s="0" t="s">
         <v>1010</v>
       </c>
-      <c r="B473" s="0" t="s">
+      <c r="C473" s="0" t="s">
         <v>1011</v>
       </c>
-      <c r="C473" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D473" s="0">
-        <v>1297</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="474">
@@ -10045,7 +10051,7 @@
         <v>52</v>
       </c>
       <c r="D474" s="0">
-        <v>298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="475">
@@ -10059,7 +10065,7 @@
         <v>52</v>
       </c>
       <c r="D475" s="0">
-        <v>596</v>
+        <v>298</v>
       </c>
     </row>
     <row r="476">
@@ -10070,10 +10076,10 @@
         <v>1017</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>384</v>
+        <v>52</v>
       </c>
       <c r="D476" s="0">
-        <v>65142.6</v>
+        <v>596</v>
       </c>
     </row>
     <row r="477">
@@ -10087,7 +10093,7 @@
         <v>384</v>
       </c>
       <c r="D477" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="478">
@@ -10098,10 +10104,10 @@
         <v>1021</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>28</v>
+        <v>384</v>
       </c>
       <c r="D478" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="479">
@@ -10112,10 +10118,10 @@
         <v>1023</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D479" s="0">
-        <v>12000</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="480">
@@ -10129,7 +10135,7 @@
         <v>52</v>
       </c>
       <c r="D480" s="0">
-        <v>17425</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="481">
@@ -10140,66 +10146,66 @@
         <v>1027</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>1028</v>
+        <v>52</v>
       </c>
       <c r="D481" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="0" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B482" s="0" t="s">
         <v>1029</v>
       </c>
-      <c r="B482" s="0" t="s">
+      <c r="C482" s="0" t="s">
         <v>1030</v>
       </c>
-      <c r="C482" s="0" t="s">
-        <v>1031</v>
-      </c>
       <c r="D482" s="0">
-        <v>2282.3</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="0" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B483" s="0" t="s">
         <v>1032</v>
       </c>
-      <c r="B483" s="0" t="s">
+      <c r="C483" s="0" t="s">
         <v>1033</v>
       </c>
-      <c r="C483" s="0" t="s">
-        <v>1034</v>
-      </c>
       <c r="D483" s="0">
-        <v>386</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B484" s="0" t="s">
         <v>1035</v>
       </c>
-      <c r="B484" s="0" t="s">
+      <c r="C484" s="0" t="s">
         <v>1036</v>
       </c>
-      <c r="C484" s="0" t="s">
-        <v>1037</v>
-      </c>
       <c r="D484" s="0">
-        <v>385.4</v>
+        <v>386</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B485" s="0" t="s">
         <v>1038</v>
       </c>
-      <c r="B485" s="0" t="s">
+      <c r="C485" s="0" t="s">
         <v>1039</v>
       </c>
-      <c r="C485" s="0" t="s">
-        <v>97</v>
-      </c>
       <c r="D485" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="486">
@@ -10210,10 +10216,10 @@
         <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="D486" s="0">
-        <v>1890</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="487">
@@ -10224,10 +10230,10 @@
         <v>1043</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>604</v>
+        <v>128</v>
       </c>
       <c r="D487" s="0">
-        <v>83000</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="488">
@@ -10238,10 +10244,10 @@
         <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>145</v>
+        <v>604</v>
       </c>
       <c r="D488" s="0">
-        <v>99</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="489">
@@ -10252,10 +10258,10 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="D489" s="0">
-        <v>950</v>
+        <v>99</v>
       </c>
     </row>
     <row r="490">
@@ -10266,10 +10272,10 @@
         <v>1049</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>479</v>
+        <v>75</v>
       </c>
       <c r="D490" s="0">
-        <v>398107</v>
+        <v>950</v>
       </c>
     </row>
     <row r="491">
@@ -10280,10 +10286,10 @@
         <v>1051</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>165</v>
+        <v>479</v>
       </c>
       <c r="D491" s="0">
-        <v>2200</v>
+        <v>398107</v>
       </c>
     </row>
     <row r="492">
@@ -10294,10 +10300,10 @@
         <v>1053</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>212</v>
+        <v>165</v>
       </c>
       <c r="D492" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="493">
@@ -10308,10 +10314,10 @@
         <v>1055</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>75</v>
+        <v>212</v>
       </c>
       <c r="D493" s="0">
-        <v>5790</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="494">
@@ -10322,10 +10328,10 @@
         <v>1057</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>952</v>
+        <v>75</v>
       </c>
       <c r="D494" s="0">
-        <v>880</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="495">
@@ -10336,7 +10342,7 @@
         <v>1059</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D495" s="0">
         <v>880</v>
@@ -10350,7 +10356,7 @@
         <v>1061</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D496" s="0">
         <v>880</v>
@@ -10364,10 +10370,10 @@
         <v>1063</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>21</v>
+        <v>954</v>
       </c>
       <c r="D497" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="498">
@@ -10378,10 +10384,10 @@
         <v>1065</v>
       </c>
       <c r="C498" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D498" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="499">
@@ -10395,7 +10401,7 @@
         <v>15</v>
       </c>
       <c r="D499" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="500">
@@ -10406,10 +10412,10 @@
         <v>1069</v>
       </c>
       <c r="C500" s="0" t="s">
-        <v>289</v>
+        <v>15</v>
       </c>
       <c r="D500" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="501">
@@ -10423,7 +10429,7 @@
         <v>289</v>
       </c>
       <c r="D501" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="502">
@@ -10434,10 +10440,10 @@
         <v>1073</v>
       </c>
       <c r="C502" s="0" t="s">
-        <v>15</v>
+        <v>289</v>
       </c>
       <c r="D502" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="503">
@@ -10451,7 +10457,7 @@
         <v>15</v>
       </c>
       <c r="D503" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="504">
@@ -10462,24 +10468,24 @@
         <v>1077</v>
       </c>
       <c r="C504" s="0" t="s">
-        <v>1078</v>
+        <v>15</v>
       </c>
       <c r="D504" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="0" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B505" s="0" t="s">
         <v>1079</v>
       </c>
-      <c r="B505" s="0" t="s">
+      <c r="C505" s="0" t="s">
         <v>1080</v>
       </c>
-      <c r="C505" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D505" s="0">
-        <v>15189</v>
+        <v>1</v>
       </c>
     </row>
     <row r="506">
@@ -10490,10 +10496,10 @@
         <v>1082</v>
       </c>
       <c r="C506" s="0" t="s">
-        <v>384</v>
+        <v>28</v>
       </c>
       <c r="D506" s="0">
-        <v>3859.93</v>
+        <v>15189</v>
       </c>
     </row>
     <row r="507">
@@ -10507,7 +10513,7 @@
         <v>384</v>
       </c>
       <c r="D507" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="508">
@@ -10518,10 +10524,10 @@
         <v>1086</v>
       </c>
       <c r="C508" s="0" t="s">
-        <v>346</v>
+        <v>384</v>
       </c>
       <c r="D508" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="509">
@@ -10535,7 +10541,7 @@
         <v>346</v>
       </c>
       <c r="D509" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="510">
@@ -10546,10 +10552,10 @@
         <v>1090</v>
       </c>
       <c r="C510" s="0" t="s">
-        <v>37</v>
+        <v>346</v>
       </c>
       <c r="D510" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="511">
@@ -10560,24 +10566,24 @@
         <v>1092</v>
       </c>
       <c r="C511" s="0" t="s">
-        <v>1093</v>
+        <v>37</v>
       </c>
       <c r="D511" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="0" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B512" s="0" t="s">
         <v>1094</v>
       </c>
-      <c r="B512" s="0" t="s">
+      <c r="C512" s="0" t="s">
         <v>1095</v>
       </c>
-      <c r="C512" s="0" t="s">
-        <v>110</v>
-      </c>
       <c r="D512" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="513">
@@ -10588,10 +10594,10 @@
         <v>1097</v>
       </c>
       <c r="C513" s="0" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="D513" s="0">
-        <v>43590.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="514">
@@ -10602,10 +10608,10 @@
         <v>1099</v>
       </c>
       <c r="C514" s="0" t="s">
-        <v>479</v>
+        <v>97</v>
       </c>
       <c r="D514" s="0">
-        <v>213700</v>
+        <v>43590.25</v>
       </c>
     </row>
     <row r="515">
@@ -10616,10 +10622,10 @@
         <v>1101</v>
       </c>
       <c r="C515" s="0" t="s">
-        <v>384</v>
+        <v>479</v>
       </c>
       <c r="D515" s="0">
-        <v>77429.29</v>
+        <v>213700</v>
       </c>
     </row>
     <row r="516">
@@ -10633,7 +10639,7 @@
         <v>384</v>
       </c>
       <c r="D516" s="0">
-        <v>42913.42</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="517">
@@ -10647,7 +10653,7 @@
         <v>384</v>
       </c>
       <c r="D517" s="0">
-        <v>88806.25</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="518">
@@ -10661,7 +10667,7 @@
         <v>384</v>
       </c>
       <c r="D518" s="0">
-        <v>50781.52</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="519">
@@ -10672,10 +10678,10 @@
         <v>1109</v>
       </c>
       <c r="C519" s="0" t="s">
-        <v>21</v>
+        <v>384</v>
       </c>
       <c r="D519" s="0">
-        <v>1600</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="520">
@@ -10686,10 +10692,10 @@
         <v>1111</v>
       </c>
       <c r="C520" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D520" s="0">
-        <v>3521.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="521">
@@ -10703,7 +10709,7 @@
         <v>28</v>
       </c>
       <c r="D521" s="0">
-        <v>3987</v>
+        <v>3521.4</v>
       </c>
     </row>
     <row r="522">
@@ -10717,7 +10723,7 @@
         <v>28</v>
       </c>
       <c r="D522" s="0">
-        <v>4086.37</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="523">
@@ -10731,7 +10737,7 @@
         <v>28</v>
       </c>
       <c r="D523" s="0">
-        <v>3382.65</v>
+        <v>4086.37</v>
       </c>
     </row>
     <row r="524">
@@ -10742,10 +10748,10 @@
         <v>1119</v>
       </c>
       <c r="C524" s="0" t="s">
-        <v>165</v>
+        <v>28</v>
       </c>
       <c r="D524" s="0">
-        <v>430</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="525">
@@ -10756,9 +10762,23 @@
         <v>1121</v>
       </c>
       <c r="C525" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D525" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="0" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B526" s="0" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C526" s="0" t="s">
         <v>145</v>
       </c>
-      <c r="D525" s="0">
+      <c r="D526" s="0">
         <v>495</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados mié 28/10/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -5850,7 +5850,7 @@
         <v>386</v>
       </c>
       <c r="D172" s="0">
-        <v>55058.9</v>
+        <v>48270</v>
       </c>
     </row>
     <row r="173">
@@ -6060,7 +6060,7 @@
         <v>386</v>
       </c>
       <c r="D187" s="0">
-        <v>37527.35</v>
+        <v>38813.17</v>
       </c>
     </row>
     <row r="188">
@@ -10176,7 +10176,7 @@
         <v>386</v>
       </c>
       <c r="D481" s="0">
-        <v>65142.6</v>
+        <v>69890</v>
       </c>
     </row>
     <row r="482">
@@ -10190,7 +10190,7 @@
         <v>386</v>
       </c>
       <c r="D482" s="0">
-        <v>23482.7</v>
+        <v>25194.62</v>
       </c>
     </row>
     <row r="483">
@@ -10722,7 +10722,7 @@
         <v>386</v>
       </c>
       <c r="D520" s="0">
-        <v>77429.29</v>
+        <v>80241.15</v>
       </c>
     </row>
     <row r="521">
@@ -10736,7 +10736,7 @@
         <v>386</v>
       </c>
       <c r="D521" s="0">
-        <v>42913.42</v>
+        <v>44471.13</v>
       </c>
     </row>
     <row r="522">
@@ -10750,7 +10750,7 @@
         <v>386</v>
       </c>
       <c r="D522" s="0">
-        <v>88806.25</v>
+        <v>92031.39</v>
       </c>
     </row>
     <row r="523">
@@ -10764,7 +10764,7 @@
         <v>386</v>
       </c>
       <c r="D523" s="0">
-        <v>50781.52</v>
+        <v>52574</v>
       </c>
     </row>
     <row r="524">

</xml_diff>